<commit_message>
Carregando dados de abril/2026
</commit_message>
<xml_diff>
--- a/upload/partos-2025.xlsx
+++ b/upload/partos-2025.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9600"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="9">
   <si>
     <t>unidade</t>
   </si>
@@ -372,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E353"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1865,7 +1865,7 @@
         <v>3</v>
       </c>
       <c r="D88" s="3">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E88" s="3">
         <v>58</v>
@@ -1873,19 +1873,19 @@
     </row>
     <row r="89" spans="1:5">
       <c r="A89" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B89" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C89" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D89" s="3">
-        <v>134</v>
+        <v>111</v>
       </c>
       <c r="E89" s="3">
-        <v>72</v>
+        <v>38</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -1896,13 +1896,13 @@
         <v>2019</v>
       </c>
       <c r="C90" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D90" s="3">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="E90" s="3">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -1913,13 +1913,13 @@
         <v>2019</v>
       </c>
       <c r="C91" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D91" s="3">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E91" s="3">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -1930,13 +1930,13 @@
         <v>2019</v>
       </c>
       <c r="C92" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D92" s="3">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="E92" s="3">
-        <v>54</v>
+        <v>72</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -1947,13 +1947,13 @@
         <v>2019</v>
       </c>
       <c r="C93" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D93" s="3">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E93" s="3">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -1964,13 +1964,13 @@
         <v>2019</v>
       </c>
       <c r="C94" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D94" s="3">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E94" s="3">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -1981,13 +1981,13 @@
         <v>2019</v>
       </c>
       <c r="C95" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D95" s="3">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="E95" s="3">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -1998,13 +1998,13 @@
         <v>2019</v>
       </c>
       <c r="C96" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D96" s="3">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E96" s="3">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2015,13 +2015,13 @@
         <v>2019</v>
       </c>
       <c r="C97" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D97" s="3">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E97" s="3">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2032,13 +2032,13 @@
         <v>2019</v>
       </c>
       <c r="C98" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D98" s="3">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E98" s="3">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2049,13 +2049,13 @@
         <v>2019</v>
       </c>
       <c r="C99" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D99" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E99" s="3">
-        <v>45</v>
+        <v>57</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2066,13 +2066,13 @@
         <v>2019</v>
       </c>
       <c r="C100" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D100" s="3">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E100" s="3">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2080,16 +2080,16 @@
         <v>6</v>
       </c>
       <c r="B101" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C101" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D101" s="3">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E101" s="3">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2100,13 +2100,13 @@
         <v>2020</v>
       </c>
       <c r="C102" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D102" s="3">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E102" s="3">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2117,13 +2117,13 @@
         <v>2020</v>
       </c>
       <c r="C103" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D103" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E103" s="3">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2134,13 +2134,13 @@
         <v>2020</v>
       </c>
       <c r="C104" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D104" s="3">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E104" s="3">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2151,13 +2151,13 @@
         <v>2020</v>
       </c>
       <c r="C105" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D105" s="3">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E105" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2168,13 +2168,13 @@
         <v>2020</v>
       </c>
       <c r="C106" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D106" s="3">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E106" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2185,13 +2185,13 @@
         <v>2020</v>
       </c>
       <c r="C107" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D107" s="3">
-        <v>153</v>
+        <v>112</v>
       </c>
       <c r="E107" s="3">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2202,13 +2202,13 @@
         <v>2020</v>
       </c>
       <c r="C108" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D108" s="3">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="E108" s="3">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2219,13 +2219,13 @@
         <v>2020</v>
       </c>
       <c r="C109" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D109" s="3">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="E109" s="3">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2236,13 +2236,13 @@
         <v>2020</v>
       </c>
       <c r="C110" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D110" s="3">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E110" s="3">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2253,13 +2253,13 @@
         <v>2020</v>
       </c>
       <c r="C111" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D111" s="3">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="E111" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2270,13 +2270,13 @@
         <v>2020</v>
       </c>
       <c r="C112" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D112" s="3">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E112" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2284,16 +2284,16 @@
         <v>6</v>
       </c>
       <c r="B113" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C113" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D113" s="3">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="E113" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2304,13 +2304,13 @@
         <v>2021</v>
       </c>
       <c r="C114" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D114" s="3">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="E114" s="3">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2321,13 +2321,13 @@
         <v>2021</v>
       </c>
       <c r="C115" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D115" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E115" s="3">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2338,13 +2338,13 @@
         <v>2021</v>
       </c>
       <c r="C116" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D116" s="3">
         <v>123</v>
       </c>
       <c r="E116" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2355,13 +2355,13 @@
         <v>2021</v>
       </c>
       <c r="C117" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D117" s="3">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E117" s="3">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2372,13 +2372,13 @@
         <v>2021</v>
       </c>
       <c r="C118" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D118" s="3">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="E118" s="3">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2389,13 +2389,13 @@
         <v>2021</v>
       </c>
       <c r="C119" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D119" s="3">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E119" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2406,13 +2406,13 @@
         <v>2021</v>
       </c>
       <c r="C120" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D120" s="3">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E120" s="3">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2423,10 +2423,10 @@
         <v>2021</v>
       </c>
       <c r="C121" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D121" s="3">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="E121" s="3">
         <v>63</v>
@@ -2440,13 +2440,13 @@
         <v>2021</v>
       </c>
       <c r="C122" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D122" s="3">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E122" s="3">
-        <v>45</v>
+        <v>63</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -2457,13 +2457,13 @@
         <v>2021</v>
       </c>
       <c r="C123" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D123" s="3">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E123" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -2474,13 +2474,13 @@
         <v>2021</v>
       </c>
       <c r="C124" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D124" s="3">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="E124" s="3">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -2488,16 +2488,16 @@
         <v>6</v>
       </c>
       <c r="B125" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C125" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D125" s="3">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="E125" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2508,13 +2508,13 @@
         <v>2022</v>
       </c>
       <c r="C126" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D126" s="3">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E126" s="3">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2525,13 +2525,13 @@
         <v>2022</v>
       </c>
       <c r="C127" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D127" s="3">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E127" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2542,13 +2542,13 @@
         <v>2022</v>
       </c>
       <c r="C128" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D128" s="3">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E128" s="3">
-        <v>52</v>
+        <v>69</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2559,10 +2559,10 @@
         <v>2022</v>
       </c>
       <c r="C129" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D129" s="3">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E129" s="3">
         <v>52</v>
@@ -2576,13 +2576,13 @@
         <v>2022</v>
       </c>
       <c r="C130" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D130" s="3">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E130" s="3">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -2593,13 +2593,13 @@
         <v>2022</v>
       </c>
       <c r="C131" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D131" s="3">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="E131" s="3">
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2610,13 +2610,13 @@
         <v>2022</v>
       </c>
       <c r="C132" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D132" s="3">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="E132" s="3">
-        <v>69</v>
+        <v>39</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2627,13 +2627,13 @@
         <v>2022</v>
       </c>
       <c r="C133" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D133" s="3">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="E133" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2644,13 +2644,13 @@
         <v>2022</v>
       </c>
       <c r="C134" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D134" s="3">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E134" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2661,13 +2661,13 @@
         <v>2022</v>
       </c>
       <c r="C135" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D135" s="3">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="E135" s="3">
-        <v>72</v>
+        <v>52</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2678,13 +2678,13 @@
         <v>2022</v>
       </c>
       <c r="C136" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D136" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E136" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2692,16 +2692,16 @@
         <v>6</v>
       </c>
       <c r="B137" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C137" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D137" s="3">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E137" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2712,13 +2712,13 @@
         <v>2023</v>
       </c>
       <c r="C138" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D138" s="3">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="E138" s="3">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2729,13 +2729,13 @@
         <v>2023</v>
       </c>
       <c r="C139" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D139" s="3">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="E139" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -2746,13 +2746,13 @@
         <v>2023</v>
       </c>
       <c r="C140" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D140" s="3">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E140" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -2763,13 +2763,13 @@
         <v>2023</v>
       </c>
       <c r="C141" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D141" s="3">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="E141" s="3">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -2780,13 +2780,13 @@
         <v>2023</v>
       </c>
       <c r="C142" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D142" s="3">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="E142" s="3">
-        <v>73</v>
+        <v>59</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -2797,13 +2797,13 @@
         <v>2023</v>
       </c>
       <c r="C143" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D143" s="3">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="E143" s="3">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -2814,13 +2814,13 @@
         <v>2023</v>
       </c>
       <c r="C144" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D144" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E144" s="3">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -2831,13 +2831,13 @@
         <v>2023</v>
       </c>
       <c r="C145" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D145" s="3">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E145" s="3">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -2848,13 +2848,13 @@
         <v>2023</v>
       </c>
       <c r="C146" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D146" s="3">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="E146" s="3">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -2865,13 +2865,13 @@
         <v>2023</v>
       </c>
       <c r="C147" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D147" s="3">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="E147" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -2882,13 +2882,13 @@
         <v>2023</v>
       </c>
       <c r="C148" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D148" s="3">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="E148" s="3">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -2896,16 +2896,16 @@
         <v>6</v>
       </c>
       <c r="B149" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C149" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D149" s="3">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="E149" s="3">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -2916,13 +2916,13 @@
         <v>2024</v>
       </c>
       <c r="C150" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D150" s="3">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="E150" s="3">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -2933,13 +2933,13 @@
         <v>2024</v>
       </c>
       <c r="C151" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D151" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E151" s="3">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -2950,13 +2950,13 @@
         <v>2024</v>
       </c>
       <c r="C152" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D152" s="3">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="E152" s="3">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -2967,13 +2967,13 @@
         <v>2024</v>
       </c>
       <c r="C153" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D153" s="3">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="E153" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -2984,13 +2984,13 @@
         <v>2024</v>
       </c>
       <c r="C154" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D154" s="3">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E154" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -3001,13 +3001,13 @@
         <v>2024</v>
       </c>
       <c r="C155" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D155" s="3">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="E155" s="3">
-        <v>42</v>
+        <v>64</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -3018,13 +3018,13 @@
         <v>2024</v>
       </c>
       <c r="C156" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D156" s="3">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E156" s="3">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -3035,13 +3035,13 @@
         <v>2024</v>
       </c>
       <c r="C157" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D157" s="3">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="E157" s="3">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -3052,13 +3052,13 @@
         <v>2024</v>
       </c>
       <c r="C158" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D158" s="3">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E158" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -3069,13 +3069,13 @@
         <v>2024</v>
       </c>
       <c r="C159" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D159" s="3">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E159" s="3">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -3086,13 +3086,13 @@
         <v>2024</v>
       </c>
       <c r="C160" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D160" s="3">
-        <v>126</v>
+        <v>90</v>
       </c>
       <c r="E160" s="3">
-        <v>62</v>
+        <v>47</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -3100,16 +3100,16 @@
         <v>6</v>
       </c>
       <c r="B161" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C161" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D161" s="3">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E161" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -3120,13 +3120,13 @@
         <v>2025</v>
       </c>
       <c r="C162" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D162" s="3">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="E162" s="3">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -3137,13 +3137,13 @@
         <v>2025</v>
       </c>
       <c r="C163" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D163" s="3">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E163" s="3">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -3154,13 +3154,13 @@
         <v>2025</v>
       </c>
       <c r="C164" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D164" s="3">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E164" s="3">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -3171,13 +3171,13 @@
         <v>2025</v>
       </c>
       <c r="C165" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D165" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E165" s="3">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -3188,13 +3188,13 @@
         <v>2025</v>
       </c>
       <c r="C166" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D166" s="3">
         <v>106</v>
       </c>
       <c r="E166" s="3">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -3205,13 +3205,13 @@
         <v>2025</v>
       </c>
       <c r="C167" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D167" s="3">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E167" s="3">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -3222,13 +3222,13 @@
         <v>2025</v>
       </c>
       <c r="C168" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D168" s="3">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="E168" s="3">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -3239,13 +3239,13 @@
         <v>2025</v>
       </c>
       <c r="C169" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D169" s="3">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E169" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -3256,13 +3256,13 @@
         <v>2025</v>
       </c>
       <c r="C170" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D170" s="3">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="E170" s="3">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -3273,13 +3273,13 @@
         <v>2025</v>
       </c>
       <c r="C171" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D171" s="3">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="E171" s="3">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -3290,13 +3290,13 @@
         <v>2025</v>
       </c>
       <c r="C172" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D172" s="3">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E172" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -3304,16 +3304,16 @@
         <v>6</v>
       </c>
       <c r="B173" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C173" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D173" s="3">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="E173" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -3324,13 +3324,13 @@
         <v>2026</v>
       </c>
       <c r="C174" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D174" s="3">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E174" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -3341,47 +3341,47 @@
         <v>2026</v>
       </c>
       <c r="C175" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D175" s="3">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E175" s="3">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="176" spans="1:5">
       <c r="A176" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B176" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C176" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D176" s="3">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E176" s="3">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="177" spans="1:5">
       <c r="A177" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B177" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C177" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D177" s="3">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="E177" s="3">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -3392,13 +3392,13 @@
         <v>2019</v>
       </c>
       <c r="C178" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D178" s="3">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E178" s="3">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -3409,13 +3409,13 @@
         <v>2019</v>
       </c>
       <c r="C179" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D179" s="3">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E179" s="3">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -3426,13 +3426,13 @@
         <v>2019</v>
       </c>
       <c r="C180" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D180" s="3">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E180" s="3">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -3443,13 +3443,13 @@
         <v>2019</v>
       </c>
       <c r="C181" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D181" s="3">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="E181" s="3">
-        <v>47</v>
+        <v>64</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -3460,13 +3460,13 @@
         <v>2019</v>
       </c>
       <c r="C182" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D182" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E182" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -3477,13 +3477,13 @@
         <v>2019</v>
       </c>
       <c r="C183" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D183" s="3">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="E183" s="3">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -3494,10 +3494,10 @@
         <v>2019</v>
       </c>
       <c r="C184" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D184" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E184" s="3">
         <v>50</v>
@@ -3511,13 +3511,13 @@
         <v>2019</v>
       </c>
       <c r="C185" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D185" s="3">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E185" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -3528,13 +3528,13 @@
         <v>2019</v>
       </c>
       <c r="C186" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D186" s="3">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E186" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -3545,13 +3545,13 @@
         <v>2019</v>
       </c>
       <c r="C187" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D187" s="3">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E187" s="3">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -3559,16 +3559,16 @@
         <v>7</v>
       </c>
       <c r="B188" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C188" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D188" s="3">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E188" s="3">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -3576,16 +3576,16 @@
         <v>7</v>
       </c>
       <c r="B189" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C189" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D189" s="3">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E189" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -3596,13 +3596,13 @@
         <v>2020</v>
       </c>
       <c r="C190" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D190" s="3">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="E190" s="3">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -3613,13 +3613,13 @@
         <v>2020</v>
       </c>
       <c r="C191" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D191" s="3">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="E191" s="3">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -3630,13 +3630,13 @@
         <v>2020</v>
       </c>
       <c r="C192" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D192" s="3">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E192" s="3">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -3647,10 +3647,10 @@
         <v>2020</v>
       </c>
       <c r="C193" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D193" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E193" s="3">
         <v>51</v>
@@ -3664,13 +3664,13 @@
         <v>2020</v>
       </c>
       <c r="C194" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D194" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E194" s="3">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -3681,13 +3681,13 @@
         <v>2020</v>
       </c>
       <c r="C195" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D195" s="3">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E195" s="3">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -3698,13 +3698,13 @@
         <v>2020</v>
       </c>
       <c r="C196" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D196" s="3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E196" s="3">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -3715,13 +3715,13 @@
         <v>2020</v>
       </c>
       <c r="C197" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D197" s="3">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="E197" s="3">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -3732,13 +3732,13 @@
         <v>2020</v>
       </c>
       <c r="C198" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D198" s="3">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="E198" s="3">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -3749,13 +3749,13 @@
         <v>2020</v>
       </c>
       <c r="C199" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D199" s="3">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E199" s="3">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -3763,16 +3763,16 @@
         <v>7</v>
       </c>
       <c r="B200" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C200" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D200" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E200" s="3">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -3780,13 +3780,13 @@
         <v>7</v>
       </c>
       <c r="B201" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C201" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D201" s="3">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E201" s="3">
         <v>44</v>
@@ -3800,13 +3800,13 @@
         <v>2021</v>
       </c>
       <c r="C202" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D202" s="3">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E202" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -3817,13 +3817,13 @@
         <v>2021</v>
       </c>
       <c r="C203" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D203" s="3">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E203" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -3834,13 +3834,13 @@
         <v>2021</v>
       </c>
       <c r="C204" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D204" s="3">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E204" s="3">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -3851,13 +3851,13 @@
         <v>2021</v>
       </c>
       <c r="C205" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D205" s="3">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="E205" s="3">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -3868,13 +3868,13 @@
         <v>2021</v>
       </c>
       <c r="C206" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D206" s="3">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="E206" s="3">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -3885,13 +3885,13 @@
         <v>2021</v>
       </c>
       <c r="C207" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D207" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E207" s="3">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -3902,13 +3902,13 @@
         <v>2021</v>
       </c>
       <c r="C208" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D208" s="3">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="E208" s="3">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -3919,13 +3919,13 @@
         <v>2021</v>
       </c>
       <c r="C209" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D209" s="3">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E209" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -3936,13 +3936,13 @@
         <v>2021</v>
       </c>
       <c r="C210" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D210" s="3">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="E210" s="3">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -3953,13 +3953,13 @@
         <v>2021</v>
       </c>
       <c r="C211" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D211" s="3">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E211" s="3">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -3967,16 +3967,16 @@
         <v>7</v>
       </c>
       <c r="B212" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C212" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D212" s="3">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E212" s="3">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -3984,16 +3984,16 @@
         <v>7</v>
       </c>
       <c r="B213" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C213" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D213" s="3">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="E213" s="3">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -4004,13 +4004,13 @@
         <v>2022</v>
       </c>
       <c r="C214" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D214" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E214" s="3">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -4021,13 +4021,13 @@
         <v>2022</v>
       </c>
       <c r="C215" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D215" s="3">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="E215" s="3">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -4038,13 +4038,13 @@
         <v>2022</v>
       </c>
       <c r="C216" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D216" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E216" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -4055,13 +4055,13 @@
         <v>2022</v>
       </c>
       <c r="C217" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D217" s="3">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="E217" s="3">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -4072,13 +4072,13 @@
         <v>2022</v>
       </c>
       <c r="C218" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D218" s="3">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E218" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -4089,13 +4089,13 @@
         <v>2022</v>
       </c>
       <c r="C219" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D219" s="3">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E219" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -4106,13 +4106,13 @@
         <v>2022</v>
       </c>
       <c r="C220" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D220" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E220" s="3">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -4123,13 +4123,13 @@
         <v>2022</v>
       </c>
       <c r="C221" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D221" s="3">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="E221" s="3">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -4140,13 +4140,13 @@
         <v>2022</v>
       </c>
       <c r="C222" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D222" s="3">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E222" s="3">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -4157,13 +4157,13 @@
         <v>2022</v>
       </c>
       <c r="C223" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D223" s="3">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E223" s="3">
-        <v>61</v>
+        <v>33</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -4171,16 +4171,16 @@
         <v>7</v>
       </c>
       <c r="B224" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C224" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D224" s="3">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="E224" s="3">
-        <v>54</v>
+        <v>38</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -4188,16 +4188,16 @@
         <v>7</v>
       </c>
       <c r="B225" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C225" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D225" s="3">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="E225" s="3">
-        <v>44</v>
+        <v>61</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -4208,13 +4208,13 @@
         <v>2023</v>
       </c>
       <c r="C226" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D226" s="3">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="E226" s="3">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -4225,13 +4225,13 @@
         <v>2023</v>
       </c>
       <c r="C227" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D227" s="3">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="E227" s="3">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -4242,13 +4242,13 @@
         <v>2023</v>
       </c>
       <c r="C228" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D228" s="3">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E228" s="3">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -4259,13 +4259,13 @@
         <v>2023</v>
       </c>
       <c r="C229" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D229" s="3">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E229" s="3">
-        <v>65</v>
+        <v>52</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -4276,13 +4276,13 @@
         <v>2023</v>
       </c>
       <c r="C230" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D230" s="3">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E230" s="3">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -4293,13 +4293,13 @@
         <v>2023</v>
       </c>
       <c r="C231" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D231" s="3">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="E231" s="3">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -4310,13 +4310,13 @@
         <v>2023</v>
       </c>
       <c r="C232" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D232" s="3">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="E232" s="3">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -4327,13 +4327,13 @@
         <v>2023</v>
       </c>
       <c r="C233" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D233" s="3">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="E233" s="3">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -4344,10 +4344,10 @@
         <v>2023</v>
       </c>
       <c r="C234" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D234" s="3">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E234" s="3">
         <v>54</v>
@@ -4361,13 +4361,13 @@
         <v>2023</v>
       </c>
       <c r="C235" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D235" s="3">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E235" s="3">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -4375,16 +4375,16 @@
         <v>7</v>
       </c>
       <c r="B236" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C236" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D236" s="3">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E236" s="3">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -4392,16 +4392,16 @@
         <v>7</v>
       </c>
       <c r="B237" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C237" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D237" s="3">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E237" s="3">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -4412,13 +4412,13 @@
         <v>2024</v>
       </c>
       <c r="C238" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D238" s="3">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E238" s="3">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="239" spans="1:5">
@@ -4429,13 +4429,13 @@
         <v>2024</v>
       </c>
       <c r="C239" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D239" s="3">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E239" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -4446,13 +4446,13 @@
         <v>2024</v>
       </c>
       <c r="C240" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D240" s="3">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="E240" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -4463,13 +4463,13 @@
         <v>2024</v>
       </c>
       <c r="C241" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D241" s="3">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E241" s="3">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -4480,13 +4480,13 @@
         <v>2024</v>
       </c>
       <c r="C242" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D242" s="3">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E242" s="3">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -4497,13 +4497,13 @@
         <v>2024</v>
       </c>
       <c r="C243" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D243" s="3">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="E243" s="3">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="244" spans="1:5">
@@ -4514,13 +4514,13 @@
         <v>2024</v>
       </c>
       <c r="C244" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D244" s="3">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="E244" s="3">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -4531,13 +4531,13 @@
         <v>2024</v>
       </c>
       <c r="C245" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D245" s="3">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="E245" s="3">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="246" spans="1:5">
@@ -4548,13 +4548,13 @@
         <v>2024</v>
       </c>
       <c r="C246" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D246" s="3">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="E246" s="3">
-        <v>25</v>
+        <v>59</v>
       </c>
     </row>
     <row r="247" spans="1:5">
@@ -4565,13 +4565,13 @@
         <v>2024</v>
       </c>
       <c r="C247" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D247" s="3">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E247" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="248" spans="1:5">
@@ -4579,16 +4579,16 @@
         <v>7</v>
       </c>
       <c r="B248" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C248" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D248" s="3">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="E248" s="3">
-        <v>54</v>
+        <v>25</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -4596,16 +4596,16 @@
         <v>7</v>
       </c>
       <c r="B249" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C249" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D249" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E249" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="250" spans="1:5">
@@ -4616,13 +4616,13 @@
         <v>2025</v>
       </c>
       <c r="C250" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D250" s="3">
-        <v>160</v>
+        <v>113</v>
       </c>
       <c r="E250" s="3">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -4633,13 +4633,13 @@
         <v>2025</v>
       </c>
       <c r="C251" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D251" s="3">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="E251" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -4650,13 +4650,13 @@
         <v>2025</v>
       </c>
       <c r="C252" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D252" s="3">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="E252" s="3">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="253" spans="1:5">
@@ -4667,13 +4667,13 @@
         <v>2025</v>
       </c>
       <c r="C253" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D253" s="3">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E253" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="254" spans="1:5">
@@ -4684,13 +4684,13 @@
         <v>2025</v>
       </c>
       <c r="C254" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D254" s="3">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E254" s="3">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="255" spans="1:5">
@@ -4701,13 +4701,13 @@
         <v>2025</v>
       </c>
       <c r="C255" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D255" s="3">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E255" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="256" spans="1:5">
@@ -4718,13 +4718,13 @@
         <v>2025</v>
       </c>
       <c r="C256" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D256" s="3">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="E256" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="257" spans="1:5">
@@ -4735,13 +4735,13 @@
         <v>2025</v>
       </c>
       <c r="C257" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D257" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E257" s="3">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -4752,13 +4752,13 @@
         <v>2025</v>
       </c>
       <c r="C258" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D258" s="3">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="E258" s="3">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -4769,13 +4769,13 @@
         <v>2025</v>
       </c>
       <c r="C259" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D259" s="3">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="E259" s="3">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="260" spans="1:5">
@@ -4783,16 +4783,16 @@
         <v>7</v>
       </c>
       <c r="B260" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C260" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D260" s="3">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E260" s="3">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -4800,16 +4800,16 @@
         <v>7</v>
       </c>
       <c r="B261" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C261" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D261" s="3">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="E261" s="3">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="262" spans="1:5">
@@ -4820,10 +4820,10 @@
         <v>2026</v>
       </c>
       <c r="C262" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D262" s="3">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="E262" s="3">
         <v>67</v>
@@ -4831,53 +4831,53 @@
     </row>
     <row r="263" spans="1:5">
       <c r="A263" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B263" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C263" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D263" s="3">
-        <v>309</v>
+        <v>128</v>
       </c>
       <c r="E263" s="3">
-        <v>101</v>
+        <v>59</v>
       </c>
     </row>
     <row r="264" spans="1:5">
       <c r="A264" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B264" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C264" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D264" s="3">
-        <v>249</v>
+        <v>122</v>
       </c>
       <c r="E264" s="3">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="265" spans="1:5">
       <c r="A265" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B265" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C265" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D265" s="3">
-        <v>298</v>
+        <v>155</v>
       </c>
       <c r="E265" s="3">
-        <v>93</v>
+        <v>85</v>
       </c>
     </row>
     <row r="266" spans="1:5">
@@ -4888,13 +4888,13 @@
         <v>2019</v>
       </c>
       <c r="C266" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D266" s="3">
-        <v>281</v>
+        <v>309</v>
       </c>
       <c r="E266" s="3">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="267" spans="1:5">
@@ -4905,13 +4905,13 @@
         <v>2019</v>
       </c>
       <c r="C267" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D267" s="3">
-        <v>296</v>
+        <v>249</v>
       </c>
       <c r="E267" s="3">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="268" spans="1:5">
@@ -4922,13 +4922,13 @@
         <v>2019</v>
       </c>
       <c r="C268" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D268" s="3">
-        <v>253</v>
+        <v>298</v>
       </c>
       <c r="E268" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="269" spans="1:5">
@@ -4939,13 +4939,13 @@
         <v>2019</v>
       </c>
       <c r="C269" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D269" s="3">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="E269" s="3">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="270" spans="1:5">
@@ -4956,13 +4956,13 @@
         <v>2019</v>
       </c>
       <c r="C270" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D270" s="3">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="E270" s="3">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="271" spans="1:5">
@@ -4973,13 +4973,13 @@
         <v>2019</v>
       </c>
       <c r="C271" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D271" s="3">
-        <v>277</v>
+        <v>253</v>
       </c>
       <c r="E271" s="3">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="272" spans="1:5">
@@ -4990,13 +4990,13 @@
         <v>2019</v>
       </c>
       <c r="C272" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D272" s="3">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E272" s="3">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="273" spans="1:5">
@@ -5007,13 +5007,13 @@
         <v>2019</v>
       </c>
       <c r="C273" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D273" s="3">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="E273" s="3">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="274" spans="1:5">
@@ -5024,13 +5024,13 @@
         <v>2019</v>
       </c>
       <c r="C274" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D274" s="3">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="E274" s="3">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="275" spans="1:5">
@@ -5038,16 +5038,16 @@
         <v>8</v>
       </c>
       <c r="B275" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C275" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D275" s="3">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="E275" s="3">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="276" spans="1:5">
@@ -5055,16 +5055,16 @@
         <v>8</v>
       </c>
       <c r="B276" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C276" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D276" s="3">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="E276" s="3">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="277" spans="1:5">
@@ -5072,16 +5072,16 @@
         <v>8</v>
       </c>
       <c r="B277" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C277" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D277" s="3">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="E277" s="3">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="278" spans="1:5">
@@ -5092,13 +5092,13 @@
         <v>2020</v>
       </c>
       <c r="C278" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D278" s="3">
-        <v>283</v>
+        <v>257</v>
       </c>
       <c r="E278" s="3">
-        <v>101</v>
+        <v>72</v>
       </c>
     </row>
     <row r="279" spans="1:5">
@@ -5109,13 +5109,13 @@
         <v>2020</v>
       </c>
       <c r="C279" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D279" s="3">
-        <v>305</v>
+        <v>261</v>
       </c>
       <c r="E279" s="3">
-        <v>112</v>
+        <v>72</v>
       </c>
     </row>
     <row r="280" spans="1:5">
@@ -5126,13 +5126,13 @@
         <v>2020</v>
       </c>
       <c r="C280" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D280" s="3">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="E280" s="3">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="281" spans="1:5">
@@ -5143,13 +5143,13 @@
         <v>2020</v>
       </c>
       <c r="C281" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D281" s="3">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E281" s="3">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -5160,13 +5160,13 @@
         <v>2020</v>
       </c>
       <c r="C282" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D282" s="3">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="E282" s="3">
-        <v>74</v>
+        <v>112</v>
       </c>
     </row>
     <row r="283" spans="1:5">
@@ -5177,13 +5177,13 @@
         <v>2020</v>
       </c>
       <c r="C283" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D283" s="3">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="E283" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -5194,10 +5194,10 @@
         <v>2020</v>
       </c>
       <c r="C284" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D284" s="3">
-        <v>247</v>
+        <v>281</v>
       </c>
       <c r="E284" s="3">
         <v>77</v>
@@ -5211,13 +5211,13 @@
         <v>2020</v>
       </c>
       <c r="C285" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D285" s="3">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E285" s="3">
-        <v>92</v>
+        <v>74</v>
       </c>
     </row>
     <row r="286" spans="1:5">
@@ -5228,13 +5228,13 @@
         <v>2020</v>
       </c>
       <c r="C286" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D286" s="3">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="E286" s="3">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="287" spans="1:5">
@@ -5242,16 +5242,16 @@
         <v>8</v>
       </c>
       <c r="B287" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C287" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D287" s="3">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E287" s="3">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="288" spans="1:5">
@@ -5259,16 +5259,16 @@
         <v>8</v>
       </c>
       <c r="B288" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C288" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D288" s="3">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="E288" s="3">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="289" spans="1:5">
@@ -5276,16 +5276,16 @@
         <v>8</v>
       </c>
       <c r="B289" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C289" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D289" s="3">
-        <v>289</v>
+        <v>260</v>
       </c>
       <c r="E289" s="3">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="290" spans="1:5">
@@ -5296,13 +5296,13 @@
         <v>2021</v>
       </c>
       <c r="C290" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D290" s="3">
-        <v>294</v>
+        <v>255</v>
       </c>
       <c r="E290" s="3">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="291" spans="1:5">
@@ -5313,13 +5313,13 @@
         <v>2021</v>
       </c>
       <c r="C291" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D291" s="3">
-        <v>318</v>
+        <v>257</v>
       </c>
       <c r="E291" s="3">
-        <v>108</v>
+        <v>89</v>
       </c>
     </row>
     <row r="292" spans="1:5">
@@ -5330,13 +5330,13 @@
         <v>2021</v>
       </c>
       <c r="C292" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D292" s="3">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="E292" s="3">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="293" spans="1:5">
@@ -5347,13 +5347,13 @@
         <v>2021</v>
       </c>
       <c r="C293" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D293" s="3">
         <v>294</v>
       </c>
       <c r="E293" s="3">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="294" spans="1:5">
@@ -5364,13 +5364,13 @@
         <v>2021</v>
       </c>
       <c r="C294" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D294" s="3">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E294" s="3">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="295" spans="1:5">
@@ -5381,13 +5381,13 @@
         <v>2021</v>
       </c>
       <c r="C295" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D295" s="3">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="E295" s="3">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="296" spans="1:5">
@@ -5398,13 +5398,13 @@
         <v>2021</v>
       </c>
       <c r="C296" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D296" s="3">
-        <v>236</v>
+        <v>294</v>
       </c>
       <c r="E296" s="3">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="297" spans="1:5">
@@ -5415,13 +5415,13 @@
         <v>2021</v>
       </c>
       <c r="C297" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D297" s="3">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="E297" s="3">
-        <v>78</v>
+        <v>107</v>
       </c>
     </row>
     <row r="298" spans="1:5">
@@ -5432,13 +5432,13 @@
         <v>2021</v>
       </c>
       <c r="C298" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D298" s="3">
-        <v>235</v>
+        <v>277</v>
       </c>
       <c r="E298" s="3">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="299" spans="1:5">
@@ -5446,16 +5446,16 @@
         <v>8</v>
       </c>
       <c r="B299" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C299" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D299" s="3">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="E299" s="3">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="300" spans="1:5">
@@ -5463,16 +5463,16 @@
         <v>8</v>
       </c>
       <c r="B300" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C300" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D300" s="3">
-        <v>224</v>
+        <v>269</v>
       </c>
       <c r="E300" s="3">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -5480,16 +5480,16 @@
         <v>8</v>
       </c>
       <c r="B301" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C301" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D301" s="3">
-        <v>278</v>
+        <v>235</v>
       </c>
       <c r="E301" s="3">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="302" spans="1:5">
@@ -5500,13 +5500,13 @@
         <v>2022</v>
       </c>
       <c r="C302" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D302" s="3">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="E302" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="303" spans="1:5">
@@ -5517,13 +5517,13 @@
         <v>2022</v>
       </c>
       <c r="C303" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D303" s="3">
-        <v>277</v>
+        <v>224</v>
       </c>
       <c r="E303" s="3">
-        <v>88</v>
+        <v>71</v>
       </c>
     </row>
     <row r="304" spans="1:5">
@@ -5534,13 +5534,13 @@
         <v>2022</v>
       </c>
       <c r="C304" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D304" s="3">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="E304" s="3">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="305" spans="1:5">
@@ -5551,13 +5551,13 @@
         <v>2022</v>
       </c>
       <c r="C305" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D305" s="3">
-        <v>265</v>
+        <v>236</v>
       </c>
       <c r="E305" s="3">
-        <v>92</v>
+        <v>64</v>
       </c>
     </row>
     <row r="306" spans="1:5">
@@ -5568,13 +5568,13 @@
         <v>2022</v>
       </c>
       <c r="C306" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D306" s="3">
-        <v>239</v>
+        <v>277</v>
       </c>
       <c r="E306" s="3">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="307" spans="1:5">
@@ -5585,13 +5585,13 @@
         <v>2022</v>
       </c>
       <c r="C307" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D307" s="3">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="E307" s="3">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="308" spans="1:5">
@@ -5602,13 +5602,13 @@
         <v>2022</v>
       </c>
       <c r="C308" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D308" s="3">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="E308" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="309" spans="1:5">
@@ -5619,13 +5619,13 @@
         <v>2022</v>
       </c>
       <c r="C309" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D309" s="3">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E309" s="3">
-        <v>103</v>
+        <v>81</v>
       </c>
     </row>
     <row r="310" spans="1:5">
@@ -5636,13 +5636,13 @@
         <v>2022</v>
       </c>
       <c r="C310" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D310" s="3">
-        <v>281</v>
+        <v>237</v>
       </c>
       <c r="E310" s="3">
-        <v>97</v>
+        <v>80</v>
       </c>
     </row>
     <row r="311" spans="1:5">
@@ -5650,16 +5650,16 @@
         <v>8</v>
       </c>
       <c r="B311" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C311" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D311" s="3">
-        <v>274</v>
+        <v>236</v>
       </c>
       <c r="E311" s="3">
-        <v>114</v>
+        <v>93</v>
       </c>
     </row>
     <row r="312" spans="1:5">
@@ -5667,16 +5667,16 @@
         <v>8</v>
       </c>
       <c r="B312" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C312" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D312" s="3">
-        <v>270</v>
+        <v>245</v>
       </c>
       <c r="E312" s="3">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="313" spans="1:5">
@@ -5684,16 +5684,16 @@
         <v>8</v>
       </c>
       <c r="B313" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C313" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D313" s="3">
-        <v>314</v>
+        <v>281</v>
       </c>
       <c r="E313" s="3">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="314" spans="1:5">
@@ -5704,13 +5704,13 @@
         <v>2023</v>
       </c>
       <c r="C314" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D314" s="3">
-        <v>508</v>
+        <v>274</v>
       </c>
       <c r="E314" s="3">
-        <v>166</v>
+        <v>114</v>
       </c>
     </row>
     <row r="315" spans="1:5">
@@ -5721,13 +5721,13 @@
         <v>2023</v>
       </c>
       <c r="C315" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D315" s="3">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E315" s="3">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="316" spans="1:5">
@@ -5738,13 +5738,13 @@
         <v>2023</v>
       </c>
       <c r="C316" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D316" s="3">
-        <v>274</v>
+        <v>314</v>
       </c>
       <c r="E316" s="3">
-        <v>87</v>
+        <v>127</v>
       </c>
     </row>
     <row r="317" spans="1:5">
@@ -5755,13 +5755,13 @@
         <v>2023</v>
       </c>
       <c r="C317" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D317" s="3">
-        <v>257</v>
+        <v>508</v>
       </c>
       <c r="E317" s="3">
-        <v>88</v>
+        <v>166</v>
       </c>
     </row>
     <row r="318" spans="1:5">
@@ -5772,13 +5772,13 @@
         <v>2023</v>
       </c>
       <c r="C318" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D318" s="3">
-        <v>286</v>
+        <v>269</v>
       </c>
       <c r="E318" s="3">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="319" spans="1:5">
@@ -5789,13 +5789,13 @@
         <v>2023</v>
       </c>
       <c r="C319" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D319" s="3">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E319" s="3">
-        <v>112</v>
+        <v>87</v>
       </c>
     </row>
     <row r="320" spans="1:5">
@@ -5806,13 +5806,13 @@
         <v>2023</v>
       </c>
       <c r="C320" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D320" s="3">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="E320" s="3">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="321" spans="1:5">
@@ -5823,13 +5823,13 @@
         <v>2023</v>
       </c>
       <c r="C321" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D321" s="3">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="E321" s="3">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="322" spans="1:5">
@@ -5840,13 +5840,13 @@
         <v>2023</v>
       </c>
       <c r="C322" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D322" s="3">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E322" s="3">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="323" spans="1:5">
@@ -5854,16 +5854,16 @@
         <v>8</v>
       </c>
       <c r="B323" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C323" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D323" s="3">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="E323" s="3">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="324" spans="1:5">
@@ -5871,16 +5871,16 @@
         <v>8</v>
       </c>
       <c r="B324" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C324" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D324" s="3">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="E324" s="3">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="325" spans="1:5">
@@ -5888,16 +5888,16 @@
         <v>8</v>
       </c>
       <c r="B325" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C325" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D325" s="3">
-        <v>314</v>
+        <v>266</v>
       </c>
       <c r="E325" s="3">
-        <v>119</v>
+        <v>93</v>
       </c>
     </row>
     <row r="326" spans="1:5">
@@ -5908,13 +5908,13 @@
         <v>2024</v>
       </c>
       <c r="C326" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D326" s="3">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="E326" s="3">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="327" spans="1:5">
@@ -5925,13 +5925,13 @@
         <v>2024</v>
       </c>
       <c r="C327" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D327" s="3">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="E327" s="3">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="328" spans="1:5">
@@ -5942,13 +5942,13 @@
         <v>2024</v>
       </c>
       <c r="C328" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D328" s="3">
-        <v>253</v>
+        <v>314</v>
       </c>
       <c r="E328" s="3">
-        <v>99</v>
+        <v>119</v>
       </c>
     </row>
     <row r="329" spans="1:5">
@@ -5959,13 +5959,13 @@
         <v>2024</v>
       </c>
       <c r="C329" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D329" s="3">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="E329" s="3">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="330" spans="1:5">
@@ -5976,13 +5976,13 @@
         <v>2024</v>
       </c>
       <c r="C330" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D330" s="3">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="E330" s="3">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="331" spans="1:5">
@@ -5993,13 +5993,13 @@
         <v>2024</v>
       </c>
       <c r="C331" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D331" s="3">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="E331" s="3">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="332" spans="1:5">
@@ -6010,13 +6010,13 @@
         <v>2024</v>
       </c>
       <c r="C332" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D332" s="3">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E332" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="333" spans="1:5">
@@ -6027,13 +6027,13 @@
         <v>2024</v>
       </c>
       <c r="C333" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D333" s="3">
-        <v>216</v>
+        <v>254</v>
       </c>
       <c r="E333" s="3">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="334" spans="1:5">
@@ -6044,13 +6044,13 @@
         <v>2024</v>
       </c>
       <c r="C334" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D334" s="3">
-        <v>235</v>
+        <v>268</v>
       </c>
       <c r="E334" s="3">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="335" spans="1:5">
@@ -6058,16 +6058,16 @@
         <v>8</v>
       </c>
       <c r="B335" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C335" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D335" s="3">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="E335" s="3">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="336" spans="1:5">
@@ -6075,16 +6075,16 @@
         <v>8</v>
       </c>
       <c r="B336" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C336" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D336" s="3">
-        <v>244</v>
+        <v>216</v>
       </c>
       <c r="E336" s="3">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="337" spans="1:5">
@@ -6092,16 +6092,16 @@
         <v>8</v>
       </c>
       <c r="B337" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C337" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D337" s="3">
-        <v>296</v>
+        <v>235</v>
       </c>
       <c r="E337" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="338" spans="1:5">
@@ -6112,13 +6112,13 @@
         <v>2025</v>
       </c>
       <c r="C338" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D338" s="3">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="E338" s="3">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="339" spans="1:5">
@@ -6129,13 +6129,13 @@
         <v>2025</v>
       </c>
       <c r="C339" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D339" s="3">
-        <v>296</v>
+        <v>244</v>
       </c>
       <c r="E339" s="3">
-        <v>119</v>
+        <v>91</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -6146,13 +6146,13 @@
         <v>2025</v>
       </c>
       <c r="C340" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D340" s="3">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="E340" s="3">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="341" spans="1:5">
@@ -6163,13 +6163,13 @@
         <v>2025</v>
       </c>
       <c r="C341" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D341" s="3">
-        <v>255</v>
+        <v>296</v>
       </c>
       <c r="E341" s="3">
-        <v>92</v>
+        <v>113</v>
       </c>
     </row>
     <row r="342" spans="1:5">
@@ -6180,13 +6180,13 @@
         <v>2025</v>
       </c>
       <c r="C342" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D342" s="3">
-        <v>262</v>
+        <v>296</v>
       </c>
       <c r="E342" s="3">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="343" spans="1:5">
@@ -6197,13 +6197,13 @@
         <v>2025</v>
       </c>
       <c r="C343" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D343" s="3">
-        <v>248</v>
+        <v>286</v>
       </c>
       <c r="E343" s="3">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="344" spans="1:5">
@@ -6214,10 +6214,10 @@
         <v>2025</v>
       </c>
       <c r="C344" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D344" s="3">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="E344" s="3">
         <v>92</v>
@@ -6231,13 +6231,13 @@
         <v>2025</v>
       </c>
       <c r="C345" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D345" s="3">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="E345" s="3">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="346" spans="1:5">
@@ -6248,13 +6248,13 @@
         <v>2025</v>
       </c>
       <c r="C346" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D346" s="3">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E346" s="3">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="347" spans="1:5">
@@ -6262,16 +6262,16 @@
         <v>8</v>
       </c>
       <c r="B347" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C347" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D347" s="3">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="E347" s="3">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="348" spans="1:5">
@@ -6279,16 +6279,16 @@
         <v>8</v>
       </c>
       <c r="B348" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C348" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D348" s="3">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E348" s="3">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="349" spans="1:5">
@@ -6296,16 +6296,84 @@
         <v>8</v>
       </c>
       <c r="B349" s="2">
+        <v>2025</v>
+      </c>
+      <c r="C349" s="2">
+        <v>12</v>
+      </c>
+      <c r="D349" s="3">
+        <v>250</v>
+      </c>
+      <c r="E349" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="350" spans="1:5">
+      <c r="A350" t="s">
+        <v>8</v>
+      </c>
+      <c r="B350" s="2">
         <v>2026</v>
       </c>
-      <c r="C349" s="2">
+      <c r="C350" s="2">
+        <v>1</v>
+      </c>
+      <c r="D350" s="3">
+        <v>250</v>
+      </c>
+      <c r="E350" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="351" spans="1:5">
+      <c r="A351" t="s">
+        <v>8</v>
+      </c>
+      <c r="B351" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C351" s="2">
+        <v>2</v>
+      </c>
+      <c r="D351" s="3">
+        <v>252</v>
+      </c>
+      <c r="E351" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="352" spans="1:5">
+      <c r="A352" t="s">
+        <v>8</v>
+      </c>
+      <c r="B352" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C352" s="2">
         <v>3</v>
       </c>
-      <c r="D349" s="3">
+      <c r="D352" s="3">
         <v>291</v>
       </c>
-      <c r="E349" s="3">
+      <c r="E352" s="3">
         <v>101</v>
+      </c>
+    </row>
+    <row r="353" spans="1:5">
+      <c r="A353" t="s">
+        <v>8</v>
+      </c>
+      <c r="B353" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C353" s="2">
+        <v>4</v>
+      </c>
+      <c r="D353" s="3">
+        <v>268</v>
+      </c>
+      <c r="E353" s="3">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carregando dados de maio/2026
</commit_message>
<xml_diff>
--- a/upload/partos-2025.xlsx
+++ b/upload/partos-2025.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="9">
   <si>
     <t>unidade</t>
   </si>
@@ -372,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E353"/>
+  <dimension ref="A1:E357"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1890,19 +1890,19 @@
     </row>
     <row r="90" spans="1:5">
       <c r="A90" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B90" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C90" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D90" s="3">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="E90" s="3">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -1913,13 +1913,13 @@
         <v>2019</v>
       </c>
       <c r="C91" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D91" s="3">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="E91" s="3">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -1930,13 +1930,13 @@
         <v>2019</v>
       </c>
       <c r="C92" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D92" s="3">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E92" s="3">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -1947,13 +1947,13 @@
         <v>2019</v>
       </c>
       <c r="C93" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D93" s="3">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="E93" s="3">
-        <v>54</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -1964,13 +1964,13 @@
         <v>2019</v>
       </c>
       <c r="C94" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D94" s="3">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E94" s="3">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -1981,13 +1981,13 @@
         <v>2019</v>
       </c>
       <c r="C95" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D95" s="3">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E95" s="3">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -1998,13 +1998,13 @@
         <v>2019</v>
       </c>
       <c r="C96" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D96" s="3">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="E96" s="3">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2015,13 +2015,13 @@
         <v>2019</v>
       </c>
       <c r="C97" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D97" s="3">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E97" s="3">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2032,13 +2032,13 @@
         <v>2019</v>
       </c>
       <c r="C98" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D98" s="3">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E98" s="3">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2049,13 +2049,13 @@
         <v>2019</v>
       </c>
       <c r="C99" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D99" s="3">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E99" s="3">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2066,13 +2066,13 @@
         <v>2019</v>
       </c>
       <c r="C100" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D100" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E100" s="3">
-        <v>45</v>
+        <v>57</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2083,13 +2083,13 @@
         <v>2019</v>
       </c>
       <c r="C101" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D101" s="3">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E101" s="3">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2097,16 +2097,16 @@
         <v>6</v>
       </c>
       <c r="B102" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C102" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D102" s="3">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E102" s="3">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2117,13 +2117,13 @@
         <v>2020</v>
       </c>
       <c r="C103" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D103" s="3">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E103" s="3">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2134,13 +2134,13 @@
         <v>2020</v>
       </c>
       <c r="C104" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D104" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E104" s="3">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2151,13 +2151,13 @@
         <v>2020</v>
       </c>
       <c r="C105" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D105" s="3">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E105" s="3">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2168,13 +2168,13 @@
         <v>2020</v>
       </c>
       <c r="C106" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D106" s="3">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E106" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2185,13 +2185,13 @@
         <v>2020</v>
       </c>
       <c r="C107" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D107" s="3">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E107" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2202,13 +2202,13 @@
         <v>2020</v>
       </c>
       <c r="C108" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D108" s="3">
-        <v>153</v>
+        <v>112</v>
       </c>
       <c r="E108" s="3">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2219,13 +2219,13 @@
         <v>2020</v>
       </c>
       <c r="C109" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D109" s="3">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="E109" s="3">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2236,13 +2236,13 @@
         <v>2020</v>
       </c>
       <c r="C110" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D110" s="3">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="E110" s="3">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2253,13 +2253,13 @@
         <v>2020</v>
       </c>
       <c r="C111" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D111" s="3">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E111" s="3">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2270,13 +2270,13 @@
         <v>2020</v>
       </c>
       <c r="C112" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D112" s="3">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="E112" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2287,13 +2287,13 @@
         <v>2020</v>
       </c>
       <c r="C113" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D113" s="3">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E113" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2301,16 +2301,16 @@
         <v>6</v>
       </c>
       <c r="B114" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C114" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D114" s="3">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="E114" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2321,13 +2321,13 @@
         <v>2021</v>
       </c>
       <c r="C115" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D115" s="3">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="E115" s="3">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2338,13 +2338,13 @@
         <v>2021</v>
       </c>
       <c r="C116" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D116" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E116" s="3">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2355,13 +2355,13 @@
         <v>2021</v>
       </c>
       <c r="C117" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D117" s="3">
         <v>123</v>
       </c>
       <c r="E117" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2372,13 +2372,13 @@
         <v>2021</v>
       </c>
       <c r="C118" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D118" s="3">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E118" s="3">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2389,13 +2389,13 @@
         <v>2021</v>
       </c>
       <c r="C119" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D119" s="3">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="E119" s="3">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2406,13 +2406,13 @@
         <v>2021</v>
       </c>
       <c r="C120" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D120" s="3">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E120" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2423,13 +2423,13 @@
         <v>2021</v>
       </c>
       <c r="C121" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D121" s="3">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E121" s="3">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -2440,10 +2440,10 @@
         <v>2021</v>
       </c>
       <c r="C122" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D122" s="3">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="E122" s="3">
         <v>63</v>
@@ -2457,13 +2457,13 @@
         <v>2021</v>
       </c>
       <c r="C123" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D123" s="3">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E123" s="3">
-        <v>45</v>
+        <v>63</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -2474,13 +2474,13 @@
         <v>2021</v>
       </c>
       <c r="C124" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D124" s="3">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E124" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -2491,13 +2491,13 @@
         <v>2021</v>
       </c>
       <c r="C125" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D125" s="3">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="E125" s="3">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2505,16 +2505,16 @@
         <v>6</v>
       </c>
       <c r="B126" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C126" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D126" s="3">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="E126" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2525,13 +2525,13 @@
         <v>2022</v>
       </c>
       <c r="C127" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D127" s="3">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E127" s="3">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2542,13 +2542,13 @@
         <v>2022</v>
       </c>
       <c r="C128" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D128" s="3">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E128" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2559,13 +2559,13 @@
         <v>2022</v>
       </c>
       <c r="C129" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D129" s="3">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E129" s="3">
-        <v>52</v>
+        <v>69</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -2576,10 +2576,10 @@
         <v>2022</v>
       </c>
       <c r="C130" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D130" s="3">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E130" s="3">
         <v>52</v>
@@ -2593,13 +2593,13 @@
         <v>2022</v>
       </c>
       <c r="C131" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D131" s="3">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E131" s="3">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2610,13 +2610,13 @@
         <v>2022</v>
       </c>
       <c r="C132" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D132" s="3">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="E132" s="3">
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2627,13 +2627,13 @@
         <v>2022</v>
       </c>
       <c r="C133" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D133" s="3">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="E133" s="3">
-        <v>69</v>
+        <v>39</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2644,13 +2644,13 @@
         <v>2022</v>
       </c>
       <c r="C134" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D134" s="3">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="E134" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2661,13 +2661,13 @@
         <v>2022</v>
       </c>
       <c r="C135" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D135" s="3">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E135" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2678,13 +2678,13 @@
         <v>2022</v>
       </c>
       <c r="C136" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D136" s="3">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="E136" s="3">
-        <v>72</v>
+        <v>52</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2695,13 +2695,13 @@
         <v>2022</v>
       </c>
       <c r="C137" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D137" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E137" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2709,16 +2709,16 @@
         <v>6</v>
       </c>
       <c r="B138" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C138" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D138" s="3">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E138" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2729,13 +2729,13 @@
         <v>2023</v>
       </c>
       <c r="C139" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D139" s="3">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="E139" s="3">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -2746,13 +2746,13 @@
         <v>2023</v>
       </c>
       <c r="C140" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D140" s="3">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="E140" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -2763,13 +2763,13 @@
         <v>2023</v>
       </c>
       <c r="C141" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D141" s="3">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E141" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -2780,13 +2780,13 @@
         <v>2023</v>
       </c>
       <c r="C142" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D142" s="3">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="E142" s="3">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -2797,13 +2797,13 @@
         <v>2023</v>
       </c>
       <c r="C143" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D143" s="3">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="E143" s="3">
-        <v>73</v>
+        <v>59</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -2814,13 +2814,13 @@
         <v>2023</v>
       </c>
       <c r="C144" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D144" s="3">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="E144" s="3">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -2831,13 +2831,13 @@
         <v>2023</v>
       </c>
       <c r="C145" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D145" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E145" s="3">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -2848,13 +2848,13 @@
         <v>2023</v>
       </c>
       <c r="C146" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D146" s="3">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E146" s="3">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -2865,13 +2865,13 @@
         <v>2023</v>
       </c>
       <c r="C147" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D147" s="3">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="E147" s="3">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -2882,13 +2882,13 @@
         <v>2023</v>
       </c>
       <c r="C148" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D148" s="3">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="E148" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -2899,13 +2899,13 @@
         <v>2023</v>
       </c>
       <c r="C149" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D149" s="3">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="E149" s="3">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -2913,16 +2913,16 @@
         <v>6</v>
       </c>
       <c r="B150" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C150" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D150" s="3">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="E150" s="3">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -2933,13 +2933,13 @@
         <v>2024</v>
       </c>
       <c r="C151" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D151" s="3">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="E151" s="3">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -2950,13 +2950,13 @@
         <v>2024</v>
       </c>
       <c r="C152" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D152" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E152" s="3">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -2967,13 +2967,13 @@
         <v>2024</v>
       </c>
       <c r="C153" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D153" s="3">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="E153" s="3">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -2984,13 +2984,13 @@
         <v>2024</v>
       </c>
       <c r="C154" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D154" s="3">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="E154" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -3001,13 +3001,13 @@
         <v>2024</v>
       </c>
       <c r="C155" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D155" s="3">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E155" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -3018,13 +3018,13 @@
         <v>2024</v>
       </c>
       <c r="C156" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D156" s="3">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="E156" s="3">
-        <v>42</v>
+        <v>64</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -3035,13 +3035,13 @@
         <v>2024</v>
       </c>
       <c r="C157" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D157" s="3">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E157" s="3">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -3052,13 +3052,13 @@
         <v>2024</v>
       </c>
       <c r="C158" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D158" s="3">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="E158" s="3">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -3069,13 +3069,13 @@
         <v>2024</v>
       </c>
       <c r="C159" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D159" s="3">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E159" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -3086,13 +3086,13 @@
         <v>2024</v>
       </c>
       <c r="C160" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D160" s="3">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="E160" s="3">
-        <v>47</v>
+        <v>60</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -3103,13 +3103,13 @@
         <v>2024</v>
       </c>
       <c r="C161" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D161" s="3">
-        <v>126</v>
+        <v>90</v>
       </c>
       <c r="E161" s="3">
-        <v>62</v>
+        <v>47</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -3117,16 +3117,16 @@
         <v>6</v>
       </c>
       <c r="B162" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C162" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D162" s="3">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E162" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -3137,13 +3137,13 @@
         <v>2025</v>
       </c>
       <c r="C163" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D163" s="3">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="E163" s="3">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -3154,13 +3154,13 @@
         <v>2025</v>
       </c>
       <c r="C164" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D164" s="3">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E164" s="3">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -3171,13 +3171,13 @@
         <v>2025</v>
       </c>
       <c r="C165" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D165" s="3">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E165" s="3">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -3188,13 +3188,13 @@
         <v>2025</v>
       </c>
       <c r="C166" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D166" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E166" s="3">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -3205,13 +3205,13 @@
         <v>2025</v>
       </c>
       <c r="C167" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D167" s="3">
         <v>106</v>
       </c>
       <c r="E167" s="3">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -3222,13 +3222,13 @@
         <v>2025</v>
       </c>
       <c r="C168" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D168" s="3">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E168" s="3">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -3239,13 +3239,13 @@
         <v>2025</v>
       </c>
       <c r="C169" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D169" s="3">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="E169" s="3">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -3256,13 +3256,13 @@
         <v>2025</v>
       </c>
       <c r="C170" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D170" s="3">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E170" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -3273,13 +3273,13 @@
         <v>2025</v>
       </c>
       <c r="C171" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D171" s="3">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="E171" s="3">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -3290,13 +3290,13 @@
         <v>2025</v>
       </c>
       <c r="C172" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D172" s="3">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="E172" s="3">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -3307,13 +3307,13 @@
         <v>2025</v>
       </c>
       <c r="C173" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D173" s="3">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E173" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -3321,16 +3321,16 @@
         <v>6</v>
       </c>
       <c r="B174" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C174" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D174" s="3">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="E174" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -3341,13 +3341,13 @@
         <v>2026</v>
       </c>
       <c r="C175" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D175" s="3">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E175" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -3358,13 +3358,13 @@
         <v>2026</v>
       </c>
       <c r="C176" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D176" s="3">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E176" s="3">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -3375,47 +3375,47 @@
         <v>2026</v>
       </c>
       <c r="C177" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D177" s="3">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E177" s="3">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="178" spans="1:5">
       <c r="A178" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B178" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C178" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D178" s="3">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="E178" s="3">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="179" spans="1:5">
       <c r="A179" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B179" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C179" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D179" s="3">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="E179" s="3">
-        <v>52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -3426,13 +3426,13 @@
         <v>2019</v>
       </c>
       <c r="C180" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D180" s="3">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E180" s="3">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -3443,13 +3443,13 @@
         <v>2019</v>
       </c>
       <c r="C181" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D181" s="3">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E181" s="3">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -3460,13 +3460,13 @@
         <v>2019</v>
       </c>
       <c r="C182" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D182" s="3">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E182" s="3">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -3477,13 +3477,13 @@
         <v>2019</v>
       </c>
       <c r="C183" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D183" s="3">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="E183" s="3">
-        <v>47</v>
+        <v>64</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -3494,13 +3494,13 @@
         <v>2019</v>
       </c>
       <c r="C184" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D184" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E184" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -3511,13 +3511,13 @@
         <v>2019</v>
       </c>
       <c r="C185" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D185" s="3">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="E185" s="3">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -3528,10 +3528,10 @@
         <v>2019</v>
       </c>
       <c r="C186" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D186" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E186" s="3">
         <v>50</v>
@@ -3545,13 +3545,13 @@
         <v>2019</v>
       </c>
       <c r="C187" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D187" s="3">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E187" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -3562,13 +3562,13 @@
         <v>2019</v>
       </c>
       <c r="C188" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D188" s="3">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E188" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -3579,13 +3579,13 @@
         <v>2019</v>
       </c>
       <c r="C189" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D189" s="3">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E189" s="3">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -3593,16 +3593,16 @@
         <v>7</v>
       </c>
       <c r="B190" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C190" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D190" s="3">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E190" s="3">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -3610,16 +3610,16 @@
         <v>7</v>
       </c>
       <c r="B191" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C191" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D191" s="3">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E191" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -3630,13 +3630,13 @@
         <v>2020</v>
       </c>
       <c r="C192" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D192" s="3">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="E192" s="3">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -3647,13 +3647,13 @@
         <v>2020</v>
       </c>
       <c r="C193" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D193" s="3">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="E193" s="3">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -3664,13 +3664,13 @@
         <v>2020</v>
       </c>
       <c r="C194" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D194" s="3">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E194" s="3">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -3681,10 +3681,10 @@
         <v>2020</v>
       </c>
       <c r="C195" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D195" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E195" s="3">
         <v>51</v>
@@ -3698,13 +3698,13 @@
         <v>2020</v>
       </c>
       <c r="C196" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D196" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E196" s="3">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -3715,13 +3715,13 @@
         <v>2020</v>
       </c>
       <c r="C197" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D197" s="3">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E197" s="3">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -3732,13 +3732,13 @@
         <v>2020</v>
       </c>
       <c r="C198" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D198" s="3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E198" s="3">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -3749,13 +3749,13 @@
         <v>2020</v>
       </c>
       <c r="C199" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D199" s="3">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="E199" s="3">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -3766,13 +3766,13 @@
         <v>2020</v>
       </c>
       <c r="C200" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D200" s="3">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="E200" s="3">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -3783,13 +3783,13 @@
         <v>2020</v>
       </c>
       <c r="C201" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D201" s="3">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E201" s="3">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -3797,16 +3797,16 @@
         <v>7</v>
       </c>
       <c r="B202" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C202" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D202" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E202" s="3">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -3814,13 +3814,13 @@
         <v>7</v>
       </c>
       <c r="B203" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C203" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D203" s="3">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E203" s="3">
         <v>44</v>
@@ -3834,13 +3834,13 @@
         <v>2021</v>
       </c>
       <c r="C204" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D204" s="3">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E204" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -3851,13 +3851,13 @@
         <v>2021</v>
       </c>
       <c r="C205" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D205" s="3">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E205" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -3868,13 +3868,13 @@
         <v>2021</v>
       </c>
       <c r="C206" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D206" s="3">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E206" s="3">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -3885,13 +3885,13 @@
         <v>2021</v>
       </c>
       <c r="C207" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D207" s="3">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="E207" s="3">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -3902,13 +3902,13 @@
         <v>2021</v>
       </c>
       <c r="C208" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D208" s="3">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="E208" s="3">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -3919,13 +3919,13 @@
         <v>2021</v>
       </c>
       <c r="C209" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D209" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E209" s="3">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -3936,13 +3936,13 @@
         <v>2021</v>
       </c>
       <c r="C210" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D210" s="3">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="E210" s="3">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -3953,13 +3953,13 @@
         <v>2021</v>
       </c>
       <c r="C211" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D211" s="3">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E211" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -3970,13 +3970,13 @@
         <v>2021</v>
       </c>
       <c r="C212" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D212" s="3">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="E212" s="3">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -3987,13 +3987,13 @@
         <v>2021</v>
       </c>
       <c r="C213" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D213" s="3">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E213" s="3">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -4001,16 +4001,16 @@
         <v>7</v>
       </c>
       <c r="B214" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C214" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D214" s="3">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E214" s="3">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -4018,16 +4018,16 @@
         <v>7</v>
       </c>
       <c r="B215" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C215" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D215" s="3">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="E215" s="3">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -4038,13 +4038,13 @@
         <v>2022</v>
       </c>
       <c r="C216" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D216" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E216" s="3">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -4055,13 +4055,13 @@
         <v>2022</v>
       </c>
       <c r="C217" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D217" s="3">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="E217" s="3">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -4072,13 +4072,13 @@
         <v>2022</v>
       </c>
       <c r="C218" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D218" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E218" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -4089,13 +4089,13 @@
         <v>2022</v>
       </c>
       <c r="C219" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D219" s="3">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="E219" s="3">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -4106,13 +4106,13 @@
         <v>2022</v>
       </c>
       <c r="C220" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D220" s="3">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E220" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -4123,13 +4123,13 @@
         <v>2022</v>
       </c>
       <c r="C221" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D221" s="3">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E221" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -4140,13 +4140,13 @@
         <v>2022</v>
       </c>
       <c r="C222" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D222" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E222" s="3">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -4157,13 +4157,13 @@
         <v>2022</v>
       </c>
       <c r="C223" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D223" s="3">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="E223" s="3">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -4174,13 +4174,13 @@
         <v>2022</v>
       </c>
       <c r="C224" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D224" s="3">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E224" s="3">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -4191,13 +4191,13 @@
         <v>2022</v>
       </c>
       <c r="C225" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D225" s="3">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E225" s="3">
-        <v>61</v>
+        <v>33</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -4205,16 +4205,16 @@
         <v>7</v>
       </c>
       <c r="B226" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C226" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D226" s="3">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="E226" s="3">
-        <v>54</v>
+        <v>38</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -4222,16 +4222,16 @@
         <v>7</v>
       </c>
       <c r="B227" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C227" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D227" s="3">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="E227" s="3">
-        <v>44</v>
+        <v>61</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -4242,13 +4242,13 @@
         <v>2023</v>
       </c>
       <c r="C228" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D228" s="3">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="E228" s="3">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -4259,13 +4259,13 @@
         <v>2023</v>
       </c>
       <c r="C229" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D229" s="3">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="E229" s="3">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -4276,13 +4276,13 @@
         <v>2023</v>
       </c>
       <c r="C230" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D230" s="3">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E230" s="3">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -4293,13 +4293,13 @@
         <v>2023</v>
       </c>
       <c r="C231" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D231" s="3">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E231" s="3">
-        <v>65</v>
+        <v>52</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -4310,13 +4310,13 @@
         <v>2023</v>
       </c>
       <c r="C232" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D232" s="3">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E232" s="3">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -4327,13 +4327,13 @@
         <v>2023</v>
       </c>
       <c r="C233" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D233" s="3">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="E233" s="3">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -4344,13 +4344,13 @@
         <v>2023</v>
       </c>
       <c r="C234" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D234" s="3">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="E234" s="3">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -4361,13 +4361,13 @@
         <v>2023</v>
       </c>
       <c r="C235" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D235" s="3">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="E235" s="3">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -4378,10 +4378,10 @@
         <v>2023</v>
       </c>
       <c r="C236" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D236" s="3">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E236" s="3">
         <v>54</v>
@@ -4395,13 +4395,13 @@
         <v>2023</v>
       </c>
       <c r="C237" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D237" s="3">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E237" s="3">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -4409,16 +4409,16 @@
         <v>7</v>
       </c>
       <c r="B238" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C238" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D238" s="3">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E238" s="3">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="239" spans="1:5">
@@ -4426,16 +4426,16 @@
         <v>7</v>
       </c>
       <c r="B239" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C239" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D239" s="3">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E239" s="3">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -4446,13 +4446,13 @@
         <v>2024</v>
       </c>
       <c r="C240" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D240" s="3">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E240" s="3">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -4463,13 +4463,13 @@
         <v>2024</v>
       </c>
       <c r="C241" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D241" s="3">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E241" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -4480,13 +4480,13 @@
         <v>2024</v>
       </c>
       <c r="C242" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D242" s="3">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="E242" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -4497,13 +4497,13 @@
         <v>2024</v>
       </c>
       <c r="C243" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D243" s="3">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E243" s="3">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="244" spans="1:5">
@@ -4514,13 +4514,13 @@
         <v>2024</v>
       </c>
       <c r="C244" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D244" s="3">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E244" s="3">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -4531,13 +4531,13 @@
         <v>2024</v>
       </c>
       <c r="C245" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D245" s="3">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="E245" s="3">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="246" spans="1:5">
@@ -4548,13 +4548,13 @@
         <v>2024</v>
       </c>
       <c r="C246" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D246" s="3">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="E246" s="3">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="247" spans="1:5">
@@ -4565,13 +4565,13 @@
         <v>2024</v>
       </c>
       <c r="C247" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D247" s="3">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="E247" s="3">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="248" spans="1:5">
@@ -4582,13 +4582,13 @@
         <v>2024</v>
       </c>
       <c r="C248" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D248" s="3">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="E248" s="3">
-        <v>25</v>
+        <v>59</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -4599,13 +4599,13 @@
         <v>2024</v>
       </c>
       <c r="C249" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D249" s="3">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E249" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="250" spans="1:5">
@@ -4613,16 +4613,16 @@
         <v>7</v>
       </c>
       <c r="B250" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C250" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D250" s="3">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="E250" s="3">
-        <v>54</v>
+        <v>25</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -4630,16 +4630,16 @@
         <v>7</v>
       </c>
       <c r="B251" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C251" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D251" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E251" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -4650,13 +4650,13 @@
         <v>2025</v>
       </c>
       <c r="C252" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D252" s="3">
-        <v>160</v>
+        <v>113</v>
       </c>
       <c r="E252" s="3">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="253" spans="1:5">
@@ -4667,13 +4667,13 @@
         <v>2025</v>
       </c>
       <c r="C253" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D253" s="3">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="E253" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="254" spans="1:5">
@@ -4684,13 +4684,13 @@
         <v>2025</v>
       </c>
       <c r="C254" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D254" s="3">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="E254" s="3">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="255" spans="1:5">
@@ -4701,13 +4701,13 @@
         <v>2025</v>
       </c>
       <c r="C255" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D255" s="3">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E255" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="256" spans="1:5">
@@ -4718,13 +4718,13 @@
         <v>2025</v>
       </c>
       <c r="C256" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D256" s="3">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E256" s="3">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="257" spans="1:5">
@@ -4735,13 +4735,13 @@
         <v>2025</v>
       </c>
       <c r="C257" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D257" s="3">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E257" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -4752,13 +4752,13 @@
         <v>2025</v>
       </c>
       <c r="C258" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D258" s="3">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="E258" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -4769,13 +4769,13 @@
         <v>2025</v>
       </c>
       <c r="C259" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D259" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E259" s="3">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="260" spans="1:5">
@@ -4786,13 +4786,13 @@
         <v>2025</v>
       </c>
       <c r="C260" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D260" s="3">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="E260" s="3">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -4803,13 +4803,13 @@
         <v>2025</v>
       </c>
       <c r="C261" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D261" s="3">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="E261" s="3">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="262" spans="1:5">
@@ -4817,16 +4817,16 @@
         <v>7</v>
       </c>
       <c r="B262" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C262" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D262" s="3">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E262" s="3">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="263" spans="1:5">
@@ -4834,16 +4834,16 @@
         <v>7</v>
       </c>
       <c r="B263" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C263" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D263" s="3">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="E263" s="3">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="264" spans="1:5">
@@ -4854,10 +4854,10 @@
         <v>2026</v>
       </c>
       <c r="C264" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D264" s="3">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="E264" s="3">
         <v>67</v>
@@ -4871,64 +4871,64 @@
         <v>2026</v>
       </c>
       <c r="C265" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D265" s="3">
-        <v>155</v>
+        <v>128</v>
       </c>
       <c r="E265" s="3">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
     <row r="266" spans="1:5">
       <c r="A266" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B266" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C266" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D266" s="3">
-        <v>309</v>
+        <v>122</v>
       </c>
       <c r="E266" s="3">
-        <v>101</v>
+        <v>67</v>
       </c>
     </row>
     <row r="267" spans="1:5">
       <c r="A267" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B267" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C267" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D267" s="3">
-        <v>249</v>
+        <v>155</v>
       </c>
       <c r="E267" s="3">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="268" spans="1:5">
       <c r="A268" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B268" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C268" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D268" s="3">
-        <v>298</v>
+        <v>127</v>
       </c>
       <c r="E268" s="3">
-        <v>93</v>
+        <v>61</v>
       </c>
     </row>
     <row r="269" spans="1:5">
@@ -4939,13 +4939,13 @@
         <v>2019</v>
       </c>
       <c r="C269" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D269" s="3">
-        <v>281</v>
+        <v>309</v>
       </c>
       <c r="E269" s="3">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="270" spans="1:5">
@@ -4956,13 +4956,13 @@
         <v>2019</v>
       </c>
       <c r="C270" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D270" s="3">
-        <v>296</v>
+        <v>249</v>
       </c>
       <c r="E270" s="3">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="271" spans="1:5">
@@ -4973,13 +4973,13 @@
         <v>2019</v>
       </c>
       <c r="C271" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D271" s="3">
-        <v>253</v>
+        <v>298</v>
       </c>
       <c r="E271" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="272" spans="1:5">
@@ -4990,13 +4990,13 @@
         <v>2019</v>
       </c>
       <c r="C272" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D272" s="3">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="E272" s="3">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="273" spans="1:5">
@@ -5007,13 +5007,13 @@
         <v>2019</v>
       </c>
       <c r="C273" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D273" s="3">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="E273" s="3">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="274" spans="1:5">
@@ -5024,13 +5024,13 @@
         <v>2019</v>
       </c>
       <c r="C274" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D274" s="3">
-        <v>277</v>
+        <v>253</v>
       </c>
       <c r="E274" s="3">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="275" spans="1:5">
@@ -5041,13 +5041,13 @@
         <v>2019</v>
       </c>
       <c r="C275" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D275" s="3">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E275" s="3">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="276" spans="1:5">
@@ -5058,13 +5058,13 @@
         <v>2019</v>
       </c>
       <c r="C276" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D276" s="3">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="E276" s="3">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="277" spans="1:5">
@@ -5075,13 +5075,13 @@
         <v>2019</v>
       </c>
       <c r="C277" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D277" s="3">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="E277" s="3">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="278" spans="1:5">
@@ -5089,16 +5089,16 @@
         <v>8</v>
       </c>
       <c r="B278" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C278" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D278" s="3">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="E278" s="3">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="279" spans="1:5">
@@ -5106,16 +5106,16 @@
         <v>8</v>
       </c>
       <c r="B279" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C279" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D279" s="3">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="E279" s="3">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="280" spans="1:5">
@@ -5123,16 +5123,16 @@
         <v>8</v>
       </c>
       <c r="B280" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C280" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D280" s="3">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="E280" s="3">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="281" spans="1:5">
@@ -5143,13 +5143,13 @@
         <v>2020</v>
       </c>
       <c r="C281" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D281" s="3">
-        <v>283</v>
+        <v>257</v>
       </c>
       <c r="E281" s="3">
-        <v>101</v>
+        <v>72</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -5160,13 +5160,13 @@
         <v>2020</v>
       </c>
       <c r="C282" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D282" s="3">
-        <v>305</v>
+        <v>261</v>
       </c>
       <c r="E282" s="3">
-        <v>112</v>
+        <v>72</v>
       </c>
     </row>
     <row r="283" spans="1:5">
@@ -5177,13 +5177,13 @@
         <v>2020</v>
       </c>
       <c r="C283" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D283" s="3">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="E283" s="3">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -5194,13 +5194,13 @@
         <v>2020</v>
       </c>
       <c r="C284" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D284" s="3">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E284" s="3">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="285" spans="1:5">
@@ -5211,13 +5211,13 @@
         <v>2020</v>
       </c>
       <c r="C285" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D285" s="3">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="E285" s="3">
-        <v>74</v>
+        <v>112</v>
       </c>
     </row>
     <row r="286" spans="1:5">
@@ -5228,13 +5228,13 @@
         <v>2020</v>
       </c>
       <c r="C286" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D286" s="3">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="E286" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="287" spans="1:5">
@@ -5245,10 +5245,10 @@
         <v>2020</v>
       </c>
       <c r="C287" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D287" s="3">
-        <v>247</v>
+        <v>281</v>
       </c>
       <c r="E287" s="3">
         <v>77</v>
@@ -5262,13 +5262,13 @@
         <v>2020</v>
       </c>
       <c r="C288" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D288" s="3">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E288" s="3">
-        <v>92</v>
+        <v>74</v>
       </c>
     </row>
     <row r="289" spans="1:5">
@@ -5279,13 +5279,13 @@
         <v>2020</v>
       </c>
       <c r="C289" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D289" s="3">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="E289" s="3">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="290" spans="1:5">
@@ -5293,16 +5293,16 @@
         <v>8</v>
       </c>
       <c r="B290" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C290" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D290" s="3">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E290" s="3">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="291" spans="1:5">
@@ -5310,16 +5310,16 @@
         <v>8</v>
       </c>
       <c r="B291" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C291" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D291" s="3">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="E291" s="3">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="292" spans="1:5">
@@ -5327,16 +5327,16 @@
         <v>8</v>
       </c>
       <c r="B292" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C292" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D292" s="3">
-        <v>289</v>
+        <v>260</v>
       </c>
       <c r="E292" s="3">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="293" spans="1:5">
@@ -5347,13 +5347,13 @@
         <v>2021</v>
       </c>
       <c r="C293" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D293" s="3">
-        <v>294</v>
+        <v>255</v>
       </c>
       <c r="E293" s="3">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="294" spans="1:5">
@@ -5364,13 +5364,13 @@
         <v>2021</v>
       </c>
       <c r="C294" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D294" s="3">
-        <v>318</v>
+        <v>257</v>
       </c>
       <c r="E294" s="3">
-        <v>108</v>
+        <v>89</v>
       </c>
     </row>
     <row r="295" spans="1:5">
@@ -5381,13 +5381,13 @@
         <v>2021</v>
       </c>
       <c r="C295" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D295" s="3">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="E295" s="3">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="296" spans="1:5">
@@ -5398,13 +5398,13 @@
         <v>2021</v>
       </c>
       <c r="C296" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D296" s="3">
         <v>294</v>
       </c>
       <c r="E296" s="3">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="297" spans="1:5">
@@ -5415,13 +5415,13 @@
         <v>2021</v>
       </c>
       <c r="C297" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D297" s="3">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E297" s="3">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="298" spans="1:5">
@@ -5432,13 +5432,13 @@
         <v>2021</v>
       </c>
       <c r="C298" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D298" s="3">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="E298" s="3">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="299" spans="1:5">
@@ -5449,13 +5449,13 @@
         <v>2021</v>
       </c>
       <c r="C299" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D299" s="3">
-        <v>236</v>
+        <v>294</v>
       </c>
       <c r="E299" s="3">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="300" spans="1:5">
@@ -5466,13 +5466,13 @@
         <v>2021</v>
       </c>
       <c r="C300" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D300" s="3">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="E300" s="3">
-        <v>78</v>
+        <v>107</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -5483,13 +5483,13 @@
         <v>2021</v>
       </c>
       <c r="C301" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D301" s="3">
-        <v>235</v>
+        <v>277</v>
       </c>
       <c r="E301" s="3">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="302" spans="1:5">
@@ -5497,16 +5497,16 @@
         <v>8</v>
       </c>
       <c r="B302" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C302" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D302" s="3">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="E302" s="3">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="303" spans="1:5">
@@ -5514,16 +5514,16 @@
         <v>8</v>
       </c>
       <c r="B303" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C303" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D303" s="3">
-        <v>224</v>
+        <v>269</v>
       </c>
       <c r="E303" s="3">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="304" spans="1:5">
@@ -5531,16 +5531,16 @@
         <v>8</v>
       </c>
       <c r="B304" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C304" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D304" s="3">
-        <v>278</v>
+        <v>235</v>
       </c>
       <c r="E304" s="3">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="305" spans="1:5">
@@ -5551,13 +5551,13 @@
         <v>2022</v>
       </c>
       <c r="C305" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D305" s="3">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="E305" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="306" spans="1:5">
@@ -5568,13 +5568,13 @@
         <v>2022</v>
       </c>
       <c r="C306" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D306" s="3">
-        <v>277</v>
+        <v>224</v>
       </c>
       <c r="E306" s="3">
-        <v>88</v>
+        <v>71</v>
       </c>
     </row>
     <row r="307" spans="1:5">
@@ -5585,13 +5585,13 @@
         <v>2022</v>
       </c>
       <c r="C307" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D307" s="3">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="E307" s="3">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="308" spans="1:5">
@@ -5602,13 +5602,13 @@
         <v>2022</v>
       </c>
       <c r="C308" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D308" s="3">
-        <v>265</v>
+        <v>236</v>
       </c>
       <c r="E308" s="3">
-        <v>92</v>
+        <v>64</v>
       </c>
     </row>
     <row r="309" spans="1:5">
@@ -5619,13 +5619,13 @@
         <v>2022</v>
       </c>
       <c r="C309" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D309" s="3">
-        <v>239</v>
+        <v>277</v>
       </c>
       <c r="E309" s="3">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="310" spans="1:5">
@@ -5636,13 +5636,13 @@
         <v>2022</v>
       </c>
       <c r="C310" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D310" s="3">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="E310" s="3">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="311" spans="1:5">
@@ -5653,13 +5653,13 @@
         <v>2022</v>
       </c>
       <c r="C311" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D311" s="3">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="E311" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="312" spans="1:5">
@@ -5670,13 +5670,13 @@
         <v>2022</v>
       </c>
       <c r="C312" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D312" s="3">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E312" s="3">
-        <v>103</v>
+        <v>81</v>
       </c>
     </row>
     <row r="313" spans="1:5">
@@ -5687,13 +5687,13 @@
         <v>2022</v>
       </c>
       <c r="C313" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D313" s="3">
-        <v>281</v>
+        <v>237</v>
       </c>
       <c r="E313" s="3">
-        <v>97</v>
+        <v>80</v>
       </c>
     </row>
     <row r="314" spans="1:5">
@@ -5701,16 +5701,16 @@
         <v>8</v>
       </c>
       <c r="B314" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C314" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D314" s="3">
-        <v>274</v>
+        <v>236</v>
       </c>
       <c r="E314" s="3">
-        <v>114</v>
+        <v>93</v>
       </c>
     </row>
     <row r="315" spans="1:5">
@@ -5718,16 +5718,16 @@
         <v>8</v>
       </c>
       <c r="B315" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C315" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D315" s="3">
-        <v>270</v>
+        <v>245</v>
       </c>
       <c r="E315" s="3">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="316" spans="1:5">
@@ -5735,16 +5735,16 @@
         <v>8</v>
       </c>
       <c r="B316" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C316" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D316" s="3">
-        <v>314</v>
+        <v>281</v>
       </c>
       <c r="E316" s="3">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="317" spans="1:5">
@@ -5755,13 +5755,13 @@
         <v>2023</v>
       </c>
       <c r="C317" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D317" s="3">
-        <v>508</v>
+        <v>274</v>
       </c>
       <c r="E317" s="3">
-        <v>166</v>
+        <v>114</v>
       </c>
     </row>
     <row r="318" spans="1:5">
@@ -5772,13 +5772,13 @@
         <v>2023</v>
       </c>
       <c r="C318" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D318" s="3">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E318" s="3">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="319" spans="1:5">
@@ -5789,13 +5789,13 @@
         <v>2023</v>
       </c>
       <c r="C319" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D319" s="3">
-        <v>274</v>
+        <v>314</v>
       </c>
       <c r="E319" s="3">
-        <v>87</v>
+        <v>127</v>
       </c>
     </row>
     <row r="320" spans="1:5">
@@ -5806,13 +5806,13 @@
         <v>2023</v>
       </c>
       <c r="C320" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D320" s="3">
-        <v>257</v>
+        <v>508</v>
       </c>
       <c r="E320" s="3">
-        <v>88</v>
+        <v>166</v>
       </c>
     </row>
     <row r="321" spans="1:5">
@@ -5823,13 +5823,13 @@
         <v>2023</v>
       </c>
       <c r="C321" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D321" s="3">
-        <v>286</v>
+        <v>269</v>
       </c>
       <c r="E321" s="3">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="322" spans="1:5">
@@ -5840,13 +5840,13 @@
         <v>2023</v>
       </c>
       <c r="C322" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D322" s="3">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E322" s="3">
-        <v>112</v>
+        <v>87</v>
       </c>
     </row>
     <row r="323" spans="1:5">
@@ -5857,13 +5857,13 @@
         <v>2023</v>
       </c>
       <c r="C323" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D323" s="3">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="E323" s="3">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="324" spans="1:5">
@@ -5874,13 +5874,13 @@
         <v>2023</v>
       </c>
       <c r="C324" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D324" s="3">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="E324" s="3">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="325" spans="1:5">
@@ -5891,13 +5891,13 @@
         <v>2023</v>
       </c>
       <c r="C325" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D325" s="3">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E325" s="3">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="326" spans="1:5">
@@ -5905,16 +5905,16 @@
         <v>8</v>
       </c>
       <c r="B326" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C326" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D326" s="3">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="E326" s="3">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="327" spans="1:5">
@@ -5922,16 +5922,16 @@
         <v>8</v>
       </c>
       <c r="B327" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C327" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D327" s="3">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="E327" s="3">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="328" spans="1:5">
@@ -5939,16 +5939,16 @@
         <v>8</v>
       </c>
       <c r="B328" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C328" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D328" s="3">
-        <v>314</v>
+        <v>266</v>
       </c>
       <c r="E328" s="3">
-        <v>119</v>
+        <v>93</v>
       </c>
     </row>
     <row r="329" spans="1:5">
@@ -5959,13 +5959,13 @@
         <v>2024</v>
       </c>
       <c r="C329" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D329" s="3">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="E329" s="3">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="330" spans="1:5">
@@ -5976,13 +5976,13 @@
         <v>2024</v>
       </c>
       <c r="C330" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D330" s="3">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="E330" s="3">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="331" spans="1:5">
@@ -5993,13 +5993,13 @@
         <v>2024</v>
       </c>
       <c r="C331" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D331" s="3">
-        <v>253</v>
+        <v>314</v>
       </c>
       <c r="E331" s="3">
-        <v>99</v>
+        <v>119</v>
       </c>
     </row>
     <row r="332" spans="1:5">
@@ -6010,13 +6010,13 @@
         <v>2024</v>
       </c>
       <c r="C332" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D332" s="3">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="E332" s="3">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="333" spans="1:5">
@@ -6027,13 +6027,13 @@
         <v>2024</v>
       </c>
       <c r="C333" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D333" s="3">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="E333" s="3">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="334" spans="1:5">
@@ -6044,13 +6044,13 @@
         <v>2024</v>
       </c>
       <c r="C334" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D334" s="3">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="E334" s="3">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="335" spans="1:5">
@@ -6061,13 +6061,13 @@
         <v>2024</v>
       </c>
       <c r="C335" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D335" s="3">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E335" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="336" spans="1:5">
@@ -6078,13 +6078,13 @@
         <v>2024</v>
       </c>
       <c r="C336" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D336" s="3">
-        <v>216</v>
+        <v>254</v>
       </c>
       <c r="E336" s="3">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="337" spans="1:5">
@@ -6095,13 +6095,13 @@
         <v>2024</v>
       </c>
       <c r="C337" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D337" s="3">
-        <v>235</v>
+        <v>268</v>
       </c>
       <c r="E337" s="3">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="338" spans="1:5">
@@ -6109,16 +6109,16 @@
         <v>8</v>
       </c>
       <c r="B338" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C338" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D338" s="3">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="E338" s="3">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="339" spans="1:5">
@@ -6126,16 +6126,16 @@
         <v>8</v>
       </c>
       <c r="B339" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C339" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D339" s="3">
-        <v>244</v>
+        <v>216</v>
       </c>
       <c r="E339" s="3">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -6143,16 +6143,16 @@
         <v>8</v>
       </c>
       <c r="B340" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C340" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D340" s="3">
-        <v>296</v>
+        <v>235</v>
       </c>
       <c r="E340" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="341" spans="1:5">
@@ -6163,13 +6163,13 @@
         <v>2025</v>
       </c>
       <c r="C341" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D341" s="3">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="E341" s="3">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="342" spans="1:5">
@@ -6180,13 +6180,13 @@
         <v>2025</v>
       </c>
       <c r="C342" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D342" s="3">
-        <v>296</v>
+        <v>244</v>
       </c>
       <c r="E342" s="3">
-        <v>119</v>
+        <v>91</v>
       </c>
     </row>
     <row r="343" spans="1:5">
@@ -6197,13 +6197,13 @@
         <v>2025</v>
       </c>
       <c r="C343" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D343" s="3">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="E343" s="3">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="344" spans="1:5">
@@ -6214,13 +6214,13 @@
         <v>2025</v>
       </c>
       <c r="C344" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D344" s="3">
-        <v>255</v>
+        <v>296</v>
       </c>
       <c r="E344" s="3">
-        <v>92</v>
+        <v>113</v>
       </c>
     </row>
     <row r="345" spans="1:5">
@@ -6231,13 +6231,13 @@
         <v>2025</v>
       </c>
       <c r="C345" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D345" s="3">
-        <v>262</v>
+        <v>296</v>
       </c>
       <c r="E345" s="3">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="346" spans="1:5">
@@ -6248,13 +6248,13 @@
         <v>2025</v>
       </c>
       <c r="C346" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D346" s="3">
-        <v>248</v>
+        <v>286</v>
       </c>
       <c r="E346" s="3">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="347" spans="1:5">
@@ -6265,10 +6265,10 @@
         <v>2025</v>
       </c>
       <c r="C347" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D347" s="3">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="E347" s="3">
         <v>92</v>
@@ -6282,13 +6282,13 @@
         <v>2025</v>
       </c>
       <c r="C348" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D348" s="3">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="E348" s="3">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="349" spans="1:5">
@@ -6299,13 +6299,13 @@
         <v>2025</v>
       </c>
       <c r="C349" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D349" s="3">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E349" s="3">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="350" spans="1:5">
@@ -6313,16 +6313,16 @@
         <v>8</v>
       </c>
       <c r="B350" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C350" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D350" s="3">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="E350" s="3">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="351" spans="1:5">
@@ -6330,16 +6330,16 @@
         <v>8</v>
       </c>
       <c r="B351" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C351" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D351" s="3">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E351" s="3">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="352" spans="1:5">
@@ -6347,16 +6347,16 @@
         <v>8</v>
       </c>
       <c r="B352" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C352" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D352" s="3">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="E352" s="3">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="353" spans="1:5">
@@ -6367,13 +6367,81 @@
         <v>2026</v>
       </c>
       <c r="C353" s="2">
+        <v>1</v>
+      </c>
+      <c r="D353" s="3">
+        <v>250</v>
+      </c>
+      <c r="E353" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="354" spans="1:5">
+      <c r="A354" t="s">
+        <v>8</v>
+      </c>
+      <c r="B354" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C354" s="2">
+        <v>2</v>
+      </c>
+      <c r="D354" s="3">
+        <v>252</v>
+      </c>
+      <c r="E354" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="355" spans="1:5">
+      <c r="A355" t="s">
+        <v>8</v>
+      </c>
+      <c r="B355" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C355" s="2">
+        <v>3</v>
+      </c>
+      <c r="D355" s="3">
+        <v>291</v>
+      </c>
+      <c r="E355" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="356" spans="1:5">
+      <c r="A356" t="s">
+        <v>8</v>
+      </c>
+      <c r="B356" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C356" s="2">
         <v>4</v>
       </c>
-      <c r="D353" s="3">
+      <c r="D356" s="3">
         <v>268</v>
       </c>
-      <c r="E353" s="3">
+      <c r="E356" s="3">
         <v>86</v>
+      </c>
+    </row>
+    <row r="357" spans="1:5">
+      <c r="A357" t="s">
+        <v>8</v>
+      </c>
+      <c r="B357" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C357" s="2">
+        <v>5</v>
+      </c>
+      <c r="D357" s="3">
+        <v>296</v>
+      </c>
+      <c r="E357" s="3">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carregando dados de junho/2026
</commit_message>
<xml_diff>
--- a/upload/partos-2025.xlsx
+++ b/upload/partos-2025.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9600"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="9">
   <si>
     <t>unidade</t>
   </si>
@@ -372,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E357"/>
+  <dimension ref="A1:E361"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1907,19 +1907,19 @@
     </row>
     <row r="91" spans="1:5">
       <c r="A91" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B91" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C91" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D91" s="3">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E91" s="3">
-        <v>72</v>
+        <v>57</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -1930,13 +1930,13 @@
         <v>2019</v>
       </c>
       <c r="C92" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D92" s="3">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="E92" s="3">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -1947,13 +1947,13 @@
         <v>2019</v>
       </c>
       <c r="C93" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D93" s="3">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E93" s="3">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -1964,13 +1964,13 @@
         <v>2019</v>
       </c>
       <c r="C94" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D94" s="3">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="E94" s="3">
-        <v>54</v>
+        <v>72</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -1981,13 +1981,13 @@
         <v>2019</v>
       </c>
       <c r="C95" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D95" s="3">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E95" s="3">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -1998,13 +1998,13 @@
         <v>2019</v>
       </c>
       <c r="C96" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D96" s="3">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E96" s="3">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2015,13 +2015,13 @@
         <v>2019</v>
       </c>
       <c r="C97" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D97" s="3">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="E97" s="3">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2032,13 +2032,13 @@
         <v>2019</v>
       </c>
       <c r="C98" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D98" s="3">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E98" s="3">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2049,13 +2049,13 @@
         <v>2019</v>
       </c>
       <c r="C99" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D99" s="3">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E99" s="3">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2066,13 +2066,13 @@
         <v>2019</v>
       </c>
       <c r="C100" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D100" s="3">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E100" s="3">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2083,13 +2083,13 @@
         <v>2019</v>
       </c>
       <c r="C101" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D101" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E101" s="3">
-        <v>45</v>
+        <v>57</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2100,13 +2100,13 @@
         <v>2019</v>
       </c>
       <c r="C102" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D102" s="3">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E102" s="3">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2114,16 +2114,16 @@
         <v>6</v>
       </c>
       <c r="B103" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C103" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D103" s="3">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E103" s="3">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2134,13 +2134,13 @@
         <v>2020</v>
       </c>
       <c r="C104" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D104" s="3">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E104" s="3">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2151,13 +2151,13 @@
         <v>2020</v>
       </c>
       <c r="C105" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D105" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E105" s="3">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2168,13 +2168,13 @@
         <v>2020</v>
       </c>
       <c r="C106" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D106" s="3">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E106" s="3">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2185,13 +2185,13 @@
         <v>2020</v>
       </c>
       <c r="C107" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D107" s="3">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E107" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2202,13 +2202,13 @@
         <v>2020</v>
       </c>
       <c r="C108" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D108" s="3">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E108" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2219,13 +2219,13 @@
         <v>2020</v>
       </c>
       <c r="C109" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D109" s="3">
-        <v>153</v>
+        <v>112</v>
       </c>
       <c r="E109" s="3">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2236,13 +2236,13 @@
         <v>2020</v>
       </c>
       <c r="C110" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D110" s="3">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="E110" s="3">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2253,13 +2253,13 @@
         <v>2020</v>
       </c>
       <c r="C111" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D111" s="3">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="E111" s="3">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2270,13 +2270,13 @@
         <v>2020</v>
       </c>
       <c r="C112" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D112" s="3">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E112" s="3">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2287,13 +2287,13 @@
         <v>2020</v>
       </c>
       <c r="C113" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D113" s="3">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="E113" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2304,13 +2304,13 @@
         <v>2020</v>
       </c>
       <c r="C114" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D114" s="3">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E114" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2318,16 +2318,16 @@
         <v>6</v>
       </c>
       <c r="B115" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C115" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D115" s="3">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="E115" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2338,13 +2338,13 @@
         <v>2021</v>
       </c>
       <c r="C116" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D116" s="3">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="E116" s="3">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2355,13 +2355,13 @@
         <v>2021</v>
       </c>
       <c r="C117" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D117" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E117" s="3">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2372,13 +2372,13 @@
         <v>2021</v>
       </c>
       <c r="C118" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D118" s="3">
         <v>123</v>
       </c>
       <c r="E118" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2389,13 +2389,13 @@
         <v>2021</v>
       </c>
       <c r="C119" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D119" s="3">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E119" s="3">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2406,13 +2406,13 @@
         <v>2021</v>
       </c>
       <c r="C120" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D120" s="3">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="E120" s="3">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2423,13 +2423,13 @@
         <v>2021</v>
       </c>
       <c r="C121" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D121" s="3">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E121" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -2440,13 +2440,13 @@
         <v>2021</v>
       </c>
       <c r="C122" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D122" s="3">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E122" s="3">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -2457,10 +2457,10 @@
         <v>2021</v>
       </c>
       <c r="C123" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D123" s="3">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="E123" s="3">
         <v>63</v>
@@ -2474,13 +2474,13 @@
         <v>2021</v>
       </c>
       <c r="C124" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D124" s="3">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E124" s="3">
-        <v>45</v>
+        <v>63</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -2491,13 +2491,13 @@
         <v>2021</v>
       </c>
       <c r="C125" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D125" s="3">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E125" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2508,13 +2508,13 @@
         <v>2021</v>
       </c>
       <c r="C126" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D126" s="3">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="E126" s="3">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2522,16 +2522,16 @@
         <v>6</v>
       </c>
       <c r="B127" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C127" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D127" s="3">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="E127" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2542,13 +2542,13 @@
         <v>2022</v>
       </c>
       <c r="C128" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D128" s="3">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E128" s="3">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2559,13 +2559,13 @@
         <v>2022</v>
       </c>
       <c r="C129" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D129" s="3">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E129" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -2576,13 +2576,13 @@
         <v>2022</v>
       </c>
       <c r="C130" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D130" s="3">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E130" s="3">
-        <v>52</v>
+        <v>69</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -2593,10 +2593,10 @@
         <v>2022</v>
       </c>
       <c r="C131" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D131" s="3">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E131" s="3">
         <v>52</v>
@@ -2610,13 +2610,13 @@
         <v>2022</v>
       </c>
       <c r="C132" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D132" s="3">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E132" s="3">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2627,13 +2627,13 @@
         <v>2022</v>
       </c>
       <c r="C133" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D133" s="3">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="E133" s="3">
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2644,13 +2644,13 @@
         <v>2022</v>
       </c>
       <c r="C134" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D134" s="3">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="E134" s="3">
-        <v>69</v>
+        <v>39</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2661,13 +2661,13 @@
         <v>2022</v>
       </c>
       <c r="C135" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D135" s="3">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="E135" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2678,13 +2678,13 @@
         <v>2022</v>
       </c>
       <c r="C136" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D136" s="3">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E136" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2695,13 +2695,13 @@
         <v>2022</v>
       </c>
       <c r="C137" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D137" s="3">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="E137" s="3">
-        <v>72</v>
+        <v>52</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2712,13 +2712,13 @@
         <v>2022</v>
       </c>
       <c r="C138" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D138" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E138" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2726,16 +2726,16 @@
         <v>6</v>
       </c>
       <c r="B139" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C139" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D139" s="3">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E139" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -2746,13 +2746,13 @@
         <v>2023</v>
       </c>
       <c r="C140" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D140" s="3">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="E140" s="3">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -2763,13 +2763,13 @@
         <v>2023</v>
       </c>
       <c r="C141" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D141" s="3">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="E141" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -2780,13 +2780,13 @@
         <v>2023</v>
       </c>
       <c r="C142" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D142" s="3">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E142" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -2797,13 +2797,13 @@
         <v>2023</v>
       </c>
       <c r="C143" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D143" s="3">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="E143" s="3">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -2814,13 +2814,13 @@
         <v>2023</v>
       </c>
       <c r="C144" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D144" s="3">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="E144" s="3">
-        <v>73</v>
+        <v>59</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -2831,13 +2831,13 @@
         <v>2023</v>
       </c>
       <c r="C145" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D145" s="3">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="E145" s="3">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -2848,13 +2848,13 @@
         <v>2023</v>
       </c>
       <c r="C146" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D146" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E146" s="3">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -2865,13 +2865,13 @@
         <v>2023</v>
       </c>
       <c r="C147" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D147" s="3">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E147" s="3">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -2882,13 +2882,13 @@
         <v>2023</v>
       </c>
       <c r="C148" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D148" s="3">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="E148" s="3">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -2899,13 +2899,13 @@
         <v>2023</v>
       </c>
       <c r="C149" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D149" s="3">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="E149" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -2916,13 +2916,13 @@
         <v>2023</v>
       </c>
       <c r="C150" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D150" s="3">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="E150" s="3">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -2930,16 +2930,16 @@
         <v>6</v>
       </c>
       <c r="B151" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C151" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D151" s="3">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="E151" s="3">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -2950,13 +2950,13 @@
         <v>2024</v>
       </c>
       <c r="C152" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D152" s="3">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="E152" s="3">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -2967,13 +2967,13 @@
         <v>2024</v>
       </c>
       <c r="C153" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D153" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E153" s="3">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -2984,13 +2984,13 @@
         <v>2024</v>
       </c>
       <c r="C154" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D154" s="3">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="E154" s="3">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -3001,13 +3001,13 @@
         <v>2024</v>
       </c>
       <c r="C155" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D155" s="3">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="E155" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -3018,13 +3018,13 @@
         <v>2024</v>
       </c>
       <c r="C156" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D156" s="3">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E156" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -3035,13 +3035,13 @@
         <v>2024</v>
       </c>
       <c r="C157" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D157" s="3">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="E157" s="3">
-        <v>42</v>
+        <v>64</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -3052,13 +3052,13 @@
         <v>2024</v>
       </c>
       <c r="C158" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D158" s="3">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E158" s="3">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -3069,13 +3069,13 @@
         <v>2024</v>
       </c>
       <c r="C159" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D159" s="3">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="E159" s="3">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -3086,13 +3086,13 @@
         <v>2024</v>
       </c>
       <c r="C160" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D160" s="3">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E160" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -3103,13 +3103,13 @@
         <v>2024</v>
       </c>
       <c r="C161" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D161" s="3">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="E161" s="3">
-        <v>47</v>
+        <v>61</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -3120,13 +3120,13 @@
         <v>2024</v>
       </c>
       <c r="C162" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D162" s="3">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="E162" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -3134,16 +3134,16 @@
         <v>6</v>
       </c>
       <c r="B163" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C163" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D163" s="3">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="E163" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -3154,13 +3154,13 @@
         <v>2025</v>
       </c>
       <c r="C164" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D164" s="3">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="E164" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -3171,13 +3171,13 @@
         <v>2025</v>
       </c>
       <c r="C165" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D165" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E165" s="3">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -3188,13 +3188,13 @@
         <v>2025</v>
       </c>
       <c r="C166" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D166" s="3">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E166" s="3">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -3205,13 +3205,13 @@
         <v>2025</v>
       </c>
       <c r="C167" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D167" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E167" s="3">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -3222,13 +3222,13 @@
         <v>2025</v>
       </c>
       <c r="C168" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D168" s="3">
         <v>106</v>
       </c>
       <c r="E168" s="3">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -3239,13 +3239,13 @@
         <v>2025</v>
       </c>
       <c r="C169" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D169" s="3">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E169" s="3">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -3256,13 +3256,13 @@
         <v>2025</v>
       </c>
       <c r="C170" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D170" s="3">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="E170" s="3">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -3273,13 +3273,13 @@
         <v>2025</v>
       </c>
       <c r="C171" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D171" s="3">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E171" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -3290,13 +3290,13 @@
         <v>2025</v>
       </c>
       <c r="C172" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D172" s="3">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="E172" s="3">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -3307,13 +3307,13 @@
         <v>2025</v>
       </c>
       <c r="C173" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D173" s="3">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="E173" s="3">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -3324,13 +3324,13 @@
         <v>2025</v>
       </c>
       <c r="C174" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D174" s="3">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E174" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -3338,16 +3338,16 @@
         <v>6</v>
       </c>
       <c r="B175" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C175" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D175" s="3">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="E175" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -3358,13 +3358,13 @@
         <v>2026</v>
       </c>
       <c r="C176" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D176" s="3">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E176" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -3375,13 +3375,13 @@
         <v>2026</v>
       </c>
       <c r="C177" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D177" s="3">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E177" s="3">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -3392,13 +3392,13 @@
         <v>2026</v>
       </c>
       <c r="C178" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D178" s="3">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E178" s="3">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -3409,47 +3409,47 @@
         <v>2026</v>
       </c>
       <c r="C179" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D179" s="3">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="E179" s="3">
-        <v>0</v>
+        <v>48</v>
       </c>
     </row>
     <row r="180" spans="1:5">
       <c r="A180" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B180" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C180" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D180" s="3">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="E180" s="3">
-        <v>43</v>
+        <v>72</v>
       </c>
     </row>
     <row r="181" spans="1:5">
       <c r="A181" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B181" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C181" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D181" s="3">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="E181" s="3">
-        <v>52</v>
+        <v>34</v>
       </c>
     </row>
     <row r="182" spans="1:5">
@@ -3460,13 +3460,13 @@
         <v>2019</v>
       </c>
       <c r="C182" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D182" s="3">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E182" s="3">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="183" spans="1:5">
@@ -3477,13 +3477,13 @@
         <v>2019</v>
       </c>
       <c r="C183" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D183" s="3">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E183" s="3">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -3494,13 +3494,13 @@
         <v>2019</v>
       </c>
       <c r="C184" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D184" s="3">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E184" s="3">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -3511,13 +3511,13 @@
         <v>2019</v>
       </c>
       <c r="C185" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D185" s="3">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="E185" s="3">
-        <v>47</v>
+        <v>64</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -3528,13 +3528,13 @@
         <v>2019</v>
       </c>
       <c r="C186" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D186" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E186" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -3545,13 +3545,13 @@
         <v>2019</v>
       </c>
       <c r="C187" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D187" s="3">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="E187" s="3">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -3562,10 +3562,10 @@
         <v>2019</v>
       </c>
       <c r="C188" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D188" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E188" s="3">
         <v>50</v>
@@ -3579,13 +3579,13 @@
         <v>2019</v>
       </c>
       <c r="C189" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D189" s="3">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E189" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -3596,13 +3596,13 @@
         <v>2019</v>
       </c>
       <c r="C190" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D190" s="3">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E190" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="191" spans="1:5">
@@ -3613,13 +3613,13 @@
         <v>2019</v>
       </c>
       <c r="C191" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D191" s="3">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E191" s="3">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -3627,16 +3627,16 @@
         <v>7</v>
       </c>
       <c r="B192" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C192" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D192" s="3">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E192" s="3">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -3644,16 +3644,16 @@
         <v>7</v>
       </c>
       <c r="B193" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C193" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D193" s="3">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E193" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -3664,13 +3664,13 @@
         <v>2020</v>
       </c>
       <c r="C194" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D194" s="3">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="E194" s="3">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -3681,13 +3681,13 @@
         <v>2020</v>
       </c>
       <c r="C195" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D195" s="3">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="E195" s="3">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -3698,13 +3698,13 @@
         <v>2020</v>
       </c>
       <c r="C196" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D196" s="3">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E196" s="3">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -3715,10 +3715,10 @@
         <v>2020</v>
       </c>
       <c r="C197" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D197" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E197" s="3">
         <v>51</v>
@@ -3732,13 +3732,13 @@
         <v>2020</v>
       </c>
       <c r="C198" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D198" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E198" s="3">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -3749,13 +3749,13 @@
         <v>2020</v>
       </c>
       <c r="C199" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D199" s="3">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E199" s="3">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="200" spans="1:5">
@@ -3766,13 +3766,13 @@
         <v>2020</v>
       </c>
       <c r="C200" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D200" s="3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E200" s="3">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -3783,13 +3783,13 @@
         <v>2020</v>
       </c>
       <c r="C201" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D201" s="3">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="E201" s="3">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -3800,13 +3800,13 @@
         <v>2020</v>
       </c>
       <c r="C202" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D202" s="3">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="E202" s="3">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -3817,13 +3817,13 @@
         <v>2020</v>
       </c>
       <c r="C203" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D203" s="3">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E203" s="3">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -3831,16 +3831,16 @@
         <v>7</v>
       </c>
       <c r="B204" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C204" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D204" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E204" s="3">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -3848,13 +3848,13 @@
         <v>7</v>
       </c>
       <c r="B205" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C205" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D205" s="3">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E205" s="3">
         <v>44</v>
@@ -3868,13 +3868,13 @@
         <v>2021</v>
       </c>
       <c r="C206" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D206" s="3">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E206" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -3885,13 +3885,13 @@
         <v>2021</v>
       </c>
       <c r="C207" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D207" s="3">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E207" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="208" spans="1:5">
@@ -3902,13 +3902,13 @@
         <v>2021</v>
       </c>
       <c r="C208" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D208" s="3">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E208" s="3">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -3919,13 +3919,13 @@
         <v>2021</v>
       </c>
       <c r="C209" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D209" s="3">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="E209" s="3">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -3936,13 +3936,13 @@
         <v>2021</v>
       </c>
       <c r="C210" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D210" s="3">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="E210" s="3">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -3953,13 +3953,13 @@
         <v>2021</v>
       </c>
       <c r="C211" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D211" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E211" s="3">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -3970,13 +3970,13 @@
         <v>2021</v>
       </c>
       <c r="C212" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D212" s="3">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="E212" s="3">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -3987,13 +3987,13 @@
         <v>2021</v>
       </c>
       <c r="C213" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D213" s="3">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E213" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -4004,13 +4004,13 @@
         <v>2021</v>
       </c>
       <c r="C214" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D214" s="3">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="E214" s="3">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -4021,13 +4021,13 @@
         <v>2021</v>
       </c>
       <c r="C215" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D215" s="3">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E215" s="3">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -4035,16 +4035,16 @@
         <v>7</v>
       </c>
       <c r="B216" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C216" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D216" s="3">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E216" s="3">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -4052,16 +4052,16 @@
         <v>7</v>
       </c>
       <c r="B217" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C217" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D217" s="3">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="E217" s="3">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -4072,13 +4072,13 @@
         <v>2022</v>
       </c>
       <c r="C218" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D218" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E218" s="3">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -4089,13 +4089,13 @@
         <v>2022</v>
       </c>
       <c r="C219" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D219" s="3">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="E219" s="3">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -4106,13 +4106,13 @@
         <v>2022</v>
       </c>
       <c r="C220" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D220" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E220" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -4123,13 +4123,13 @@
         <v>2022</v>
       </c>
       <c r="C221" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D221" s="3">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="E221" s="3">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -4140,13 +4140,13 @@
         <v>2022</v>
       </c>
       <c r="C222" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D222" s="3">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E222" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -4157,13 +4157,13 @@
         <v>2022</v>
       </c>
       <c r="C223" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D223" s="3">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E223" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -4174,13 +4174,13 @@
         <v>2022</v>
       </c>
       <c r="C224" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D224" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E224" s="3">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -4191,13 +4191,13 @@
         <v>2022</v>
       </c>
       <c r="C225" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D225" s="3">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="E225" s="3">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -4208,13 +4208,13 @@
         <v>2022</v>
       </c>
       <c r="C226" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D226" s="3">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E226" s="3">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -4225,13 +4225,13 @@
         <v>2022</v>
       </c>
       <c r="C227" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D227" s="3">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E227" s="3">
-        <v>61</v>
+        <v>33</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -4239,16 +4239,16 @@
         <v>7</v>
       </c>
       <c r="B228" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C228" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D228" s="3">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="E228" s="3">
-        <v>54</v>
+        <v>38</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -4256,16 +4256,16 @@
         <v>7</v>
       </c>
       <c r="B229" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C229" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D229" s="3">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="E229" s="3">
-        <v>44</v>
+        <v>61</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -4276,13 +4276,13 @@
         <v>2023</v>
       </c>
       <c r="C230" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D230" s="3">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="E230" s="3">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -4293,13 +4293,13 @@
         <v>2023</v>
       </c>
       <c r="C231" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D231" s="3">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="E231" s="3">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -4310,13 +4310,13 @@
         <v>2023</v>
       </c>
       <c r="C232" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D232" s="3">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E232" s="3">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -4327,13 +4327,13 @@
         <v>2023</v>
       </c>
       <c r="C233" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D233" s="3">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E233" s="3">
-        <v>65</v>
+        <v>52</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -4344,13 +4344,13 @@
         <v>2023</v>
       </c>
       <c r="C234" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D234" s="3">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E234" s="3">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -4361,13 +4361,13 @@
         <v>2023</v>
       </c>
       <c r="C235" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D235" s="3">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="E235" s="3">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -4378,13 +4378,13 @@
         <v>2023</v>
       </c>
       <c r="C236" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D236" s="3">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="E236" s="3">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -4395,13 +4395,13 @@
         <v>2023</v>
       </c>
       <c r="C237" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D237" s="3">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="E237" s="3">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -4412,10 +4412,10 @@
         <v>2023</v>
       </c>
       <c r="C238" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D238" s="3">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E238" s="3">
         <v>54</v>
@@ -4429,13 +4429,13 @@
         <v>2023</v>
       </c>
       <c r="C239" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D239" s="3">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E239" s="3">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -4443,16 +4443,16 @@
         <v>7</v>
       </c>
       <c r="B240" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C240" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D240" s="3">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E240" s="3">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="241" spans="1:5">
@@ -4460,16 +4460,16 @@
         <v>7</v>
       </c>
       <c r="B241" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C241" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D241" s="3">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E241" s="3">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -4480,13 +4480,13 @@
         <v>2024</v>
       </c>
       <c r="C242" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D242" s="3">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E242" s="3">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -4497,13 +4497,13 @@
         <v>2024</v>
       </c>
       <c r="C243" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D243" s="3">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E243" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="244" spans="1:5">
@@ -4514,13 +4514,13 @@
         <v>2024</v>
       </c>
       <c r="C244" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D244" s="3">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="E244" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -4531,13 +4531,13 @@
         <v>2024</v>
       </c>
       <c r="C245" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D245" s="3">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E245" s="3">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="246" spans="1:5">
@@ -4548,13 +4548,13 @@
         <v>2024</v>
       </c>
       <c r="C246" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D246" s="3">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E246" s="3">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="247" spans="1:5">
@@ -4565,13 +4565,13 @@
         <v>2024</v>
       </c>
       <c r="C247" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D247" s="3">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="E247" s="3">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="248" spans="1:5">
@@ -4582,13 +4582,13 @@
         <v>2024</v>
       </c>
       <c r="C248" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D248" s="3">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="E248" s="3">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -4599,13 +4599,13 @@
         <v>2024</v>
       </c>
       <c r="C249" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D249" s="3">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="E249" s="3">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="250" spans="1:5">
@@ -4616,13 +4616,13 @@
         <v>2024</v>
       </c>
       <c r="C250" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D250" s="3">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="E250" s="3">
-        <v>25</v>
+        <v>59</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -4633,13 +4633,13 @@
         <v>2024</v>
       </c>
       <c r="C251" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D251" s="3">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E251" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -4647,16 +4647,16 @@
         <v>7</v>
       </c>
       <c r="B252" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C252" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D252" s="3">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="E252" s="3">
-        <v>54</v>
+        <v>25</v>
       </c>
     </row>
     <row r="253" spans="1:5">
@@ -4664,16 +4664,16 @@
         <v>7</v>
       </c>
       <c r="B253" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C253" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D253" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E253" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="254" spans="1:5">
@@ -4684,13 +4684,13 @@
         <v>2025</v>
       </c>
       <c r="C254" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D254" s="3">
-        <v>160</v>
+        <v>113</v>
       </c>
       <c r="E254" s="3">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="255" spans="1:5">
@@ -4701,13 +4701,13 @@
         <v>2025</v>
       </c>
       <c r="C255" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D255" s="3">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="E255" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="256" spans="1:5">
@@ -4718,13 +4718,13 @@
         <v>2025</v>
       </c>
       <c r="C256" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D256" s="3">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="E256" s="3">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="257" spans="1:5">
@@ -4735,13 +4735,13 @@
         <v>2025</v>
       </c>
       <c r="C257" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D257" s="3">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E257" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -4752,13 +4752,13 @@
         <v>2025</v>
       </c>
       <c r="C258" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D258" s="3">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E258" s="3">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -4769,13 +4769,13 @@
         <v>2025</v>
       </c>
       <c r="C259" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D259" s="3">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E259" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="260" spans="1:5">
@@ -4786,13 +4786,13 @@
         <v>2025</v>
       </c>
       <c r="C260" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D260" s="3">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="E260" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -4803,13 +4803,13 @@
         <v>2025</v>
       </c>
       <c r="C261" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D261" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E261" s="3">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="262" spans="1:5">
@@ -4820,13 +4820,13 @@
         <v>2025</v>
       </c>
       <c r="C262" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D262" s="3">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="E262" s="3">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="263" spans="1:5">
@@ -4837,13 +4837,13 @@
         <v>2025</v>
       </c>
       <c r="C263" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D263" s="3">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="E263" s="3">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="264" spans="1:5">
@@ -4851,16 +4851,16 @@
         <v>7</v>
       </c>
       <c r="B264" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C264" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D264" s="3">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E264" s="3">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="265" spans="1:5">
@@ -4868,16 +4868,16 @@
         <v>7</v>
       </c>
       <c r="B265" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C265" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D265" s="3">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="E265" s="3">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="266" spans="1:5">
@@ -4888,10 +4888,10 @@
         <v>2026</v>
       </c>
       <c r="C266" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D266" s="3">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="E266" s="3">
         <v>67</v>
@@ -4905,13 +4905,13 @@
         <v>2026</v>
       </c>
       <c r="C267" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D267" s="3">
-        <v>155</v>
+        <v>128</v>
       </c>
       <c r="E267" s="3">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
     <row r="268" spans="1:5">
@@ -4922,64 +4922,64 @@
         <v>2026</v>
       </c>
       <c r="C268" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D268" s="3">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E268" s="3">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="269" spans="1:5">
       <c r="A269" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B269" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C269" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D269" s="3">
-        <v>309</v>
+        <v>155</v>
       </c>
       <c r="E269" s="3">
-        <v>101</v>
+        <v>85</v>
       </c>
     </row>
     <row r="270" spans="1:5">
       <c r="A270" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B270" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C270" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D270" s="3">
-        <v>249</v>
+        <v>127</v>
       </c>
       <c r="E270" s="3">
-        <v>72</v>
+        <v>61</v>
       </c>
     </row>
     <row r="271" spans="1:5">
       <c r="A271" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B271" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C271" s="2">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D271" s="3">
-        <v>298</v>
+        <v>119</v>
       </c>
       <c r="E271" s="3">
-        <v>93</v>
+        <v>66</v>
       </c>
     </row>
     <row r="272" spans="1:5">
@@ -4990,13 +4990,13 @@
         <v>2019</v>
       </c>
       <c r="C272" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D272" s="3">
-        <v>281</v>
+        <v>309</v>
       </c>
       <c r="E272" s="3">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="273" spans="1:5">
@@ -5007,13 +5007,13 @@
         <v>2019</v>
       </c>
       <c r="C273" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D273" s="3">
-        <v>296</v>
+        <v>249</v>
       </c>
       <c r="E273" s="3">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="274" spans="1:5">
@@ -5024,13 +5024,13 @@
         <v>2019</v>
       </c>
       <c r="C274" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D274" s="3">
-        <v>253</v>
+        <v>298</v>
       </c>
       <c r="E274" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="275" spans="1:5">
@@ -5041,13 +5041,13 @@
         <v>2019</v>
       </c>
       <c r="C275" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D275" s="3">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="E275" s="3">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="276" spans="1:5">
@@ -5058,13 +5058,13 @@
         <v>2019</v>
       </c>
       <c r="C276" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D276" s="3">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="E276" s="3">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="277" spans="1:5">
@@ -5075,13 +5075,13 @@
         <v>2019</v>
       </c>
       <c r="C277" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D277" s="3">
-        <v>277</v>
+        <v>253</v>
       </c>
       <c r="E277" s="3">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="278" spans="1:5">
@@ -5092,13 +5092,13 @@
         <v>2019</v>
       </c>
       <c r="C278" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D278" s="3">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E278" s="3">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="279" spans="1:5">
@@ -5109,13 +5109,13 @@
         <v>2019</v>
       </c>
       <c r="C279" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D279" s="3">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="E279" s="3">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="280" spans="1:5">
@@ -5126,13 +5126,13 @@
         <v>2019</v>
       </c>
       <c r="C280" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D280" s="3">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="E280" s="3">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="281" spans="1:5">
@@ -5140,16 +5140,16 @@
         <v>8</v>
       </c>
       <c r="B281" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C281" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D281" s="3">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="E281" s="3">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -5157,16 +5157,16 @@
         <v>8</v>
       </c>
       <c r="B282" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C282" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D282" s="3">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="E282" s="3">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="283" spans="1:5">
@@ -5174,16 +5174,16 @@
         <v>8</v>
       </c>
       <c r="B283" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C283" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D283" s="3">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="E283" s="3">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -5194,13 +5194,13 @@
         <v>2020</v>
       </c>
       <c r="C284" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D284" s="3">
-        <v>283</v>
+        <v>257</v>
       </c>
       <c r="E284" s="3">
-        <v>101</v>
+        <v>72</v>
       </c>
     </row>
     <row r="285" spans="1:5">
@@ -5211,13 +5211,13 @@
         <v>2020</v>
       </c>
       <c r="C285" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D285" s="3">
-        <v>305</v>
+        <v>261</v>
       </c>
       <c r="E285" s="3">
-        <v>112</v>
+        <v>72</v>
       </c>
     </row>
     <row r="286" spans="1:5">
@@ -5228,13 +5228,13 @@
         <v>2020</v>
       </c>
       <c r="C286" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D286" s="3">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="E286" s="3">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="287" spans="1:5">
@@ -5245,13 +5245,13 @@
         <v>2020</v>
       </c>
       <c r="C287" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D287" s="3">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E287" s="3">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="288" spans="1:5">
@@ -5262,13 +5262,13 @@
         <v>2020</v>
       </c>
       <c r="C288" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D288" s="3">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="E288" s="3">
-        <v>74</v>
+        <v>112</v>
       </c>
     </row>
     <row r="289" spans="1:5">
@@ -5279,13 +5279,13 @@
         <v>2020</v>
       </c>
       <c r="C289" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D289" s="3">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="E289" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="290" spans="1:5">
@@ -5296,10 +5296,10 @@
         <v>2020</v>
       </c>
       <c r="C290" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D290" s="3">
-        <v>247</v>
+        <v>281</v>
       </c>
       <c r="E290" s="3">
         <v>77</v>
@@ -5313,13 +5313,13 @@
         <v>2020</v>
       </c>
       <c r="C291" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D291" s="3">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E291" s="3">
-        <v>92</v>
+        <v>74</v>
       </c>
     </row>
     <row r="292" spans="1:5">
@@ -5330,13 +5330,13 @@
         <v>2020</v>
       </c>
       <c r="C292" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D292" s="3">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="E292" s="3">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="293" spans="1:5">
@@ -5344,16 +5344,16 @@
         <v>8</v>
       </c>
       <c r="B293" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C293" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D293" s="3">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E293" s="3">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="294" spans="1:5">
@@ -5361,16 +5361,16 @@
         <v>8</v>
       </c>
       <c r="B294" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C294" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D294" s="3">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="E294" s="3">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="295" spans="1:5">
@@ -5378,16 +5378,16 @@
         <v>8</v>
       </c>
       <c r="B295" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C295" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D295" s="3">
-        <v>289</v>
+        <v>260</v>
       </c>
       <c r="E295" s="3">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="296" spans="1:5">
@@ -5398,13 +5398,13 @@
         <v>2021</v>
       </c>
       <c r="C296" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D296" s="3">
-        <v>294</v>
+        <v>255</v>
       </c>
       <c r="E296" s="3">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="297" spans="1:5">
@@ -5415,13 +5415,13 @@
         <v>2021</v>
       </c>
       <c r="C297" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D297" s="3">
-        <v>318</v>
+        <v>257</v>
       </c>
       <c r="E297" s="3">
-        <v>108</v>
+        <v>89</v>
       </c>
     </row>
     <row r="298" spans="1:5">
@@ -5432,13 +5432,13 @@
         <v>2021</v>
       </c>
       <c r="C298" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D298" s="3">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="E298" s="3">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="299" spans="1:5">
@@ -5449,13 +5449,13 @@
         <v>2021</v>
       </c>
       <c r="C299" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D299" s="3">
         <v>294</v>
       </c>
       <c r="E299" s="3">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="300" spans="1:5">
@@ -5466,13 +5466,13 @@
         <v>2021</v>
       </c>
       <c r="C300" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D300" s="3">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E300" s="3">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -5483,13 +5483,13 @@
         <v>2021</v>
       </c>
       <c r="C301" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D301" s="3">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="E301" s="3">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="302" spans="1:5">
@@ -5500,13 +5500,13 @@
         <v>2021</v>
       </c>
       <c r="C302" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D302" s="3">
-        <v>236</v>
+        <v>294</v>
       </c>
       <c r="E302" s="3">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="303" spans="1:5">
@@ -5517,13 +5517,13 @@
         <v>2021</v>
       </c>
       <c r="C303" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D303" s="3">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="E303" s="3">
-        <v>78</v>
+        <v>107</v>
       </c>
     </row>
     <row r="304" spans="1:5">
@@ -5534,13 +5534,13 @@
         <v>2021</v>
       </c>
       <c r="C304" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D304" s="3">
-        <v>235</v>
+        <v>277</v>
       </c>
       <c r="E304" s="3">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="305" spans="1:5">
@@ -5548,16 +5548,16 @@
         <v>8</v>
       </c>
       <c r="B305" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C305" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D305" s="3">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="E305" s="3">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="306" spans="1:5">
@@ -5565,16 +5565,16 @@
         <v>8</v>
       </c>
       <c r="B306" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C306" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D306" s="3">
-        <v>224</v>
+        <v>269</v>
       </c>
       <c r="E306" s="3">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="307" spans="1:5">
@@ -5582,16 +5582,16 @@
         <v>8</v>
       </c>
       <c r="B307" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C307" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D307" s="3">
-        <v>278</v>
+        <v>235</v>
       </c>
       <c r="E307" s="3">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="308" spans="1:5">
@@ -5602,13 +5602,13 @@
         <v>2022</v>
       </c>
       <c r="C308" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D308" s="3">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="E308" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="309" spans="1:5">
@@ -5619,13 +5619,13 @@
         <v>2022</v>
       </c>
       <c r="C309" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D309" s="3">
-        <v>277</v>
+        <v>224</v>
       </c>
       <c r="E309" s="3">
-        <v>88</v>
+        <v>71</v>
       </c>
     </row>
     <row r="310" spans="1:5">
@@ -5636,13 +5636,13 @@
         <v>2022</v>
       </c>
       <c r="C310" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D310" s="3">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="E310" s="3">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="311" spans="1:5">
@@ -5653,13 +5653,13 @@
         <v>2022</v>
       </c>
       <c r="C311" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D311" s="3">
-        <v>265</v>
+        <v>236</v>
       </c>
       <c r="E311" s="3">
-        <v>92</v>
+        <v>64</v>
       </c>
     </row>
     <row r="312" spans="1:5">
@@ -5670,13 +5670,13 @@
         <v>2022</v>
       </c>
       <c r="C312" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D312" s="3">
-        <v>239</v>
+        <v>277</v>
       </c>
       <c r="E312" s="3">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="313" spans="1:5">
@@ -5687,13 +5687,13 @@
         <v>2022</v>
       </c>
       <c r="C313" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D313" s="3">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="E313" s="3">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="314" spans="1:5">
@@ -5704,13 +5704,13 @@
         <v>2022</v>
       </c>
       <c r="C314" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D314" s="3">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="E314" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="315" spans="1:5">
@@ -5721,13 +5721,13 @@
         <v>2022</v>
       </c>
       <c r="C315" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D315" s="3">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E315" s="3">
-        <v>103</v>
+        <v>81</v>
       </c>
     </row>
     <row r="316" spans="1:5">
@@ -5738,13 +5738,13 @@
         <v>2022</v>
       </c>
       <c r="C316" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D316" s="3">
-        <v>281</v>
+        <v>237</v>
       </c>
       <c r="E316" s="3">
-        <v>97</v>
+        <v>80</v>
       </c>
     </row>
     <row r="317" spans="1:5">
@@ -5752,16 +5752,16 @@
         <v>8</v>
       </c>
       <c r="B317" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C317" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D317" s="3">
-        <v>274</v>
+        <v>236</v>
       </c>
       <c r="E317" s="3">
-        <v>114</v>
+        <v>93</v>
       </c>
     </row>
     <row r="318" spans="1:5">
@@ -5769,16 +5769,16 @@
         <v>8</v>
       </c>
       <c r="B318" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C318" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D318" s="3">
-        <v>270</v>
+        <v>245</v>
       </c>
       <c r="E318" s="3">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="319" spans="1:5">
@@ -5786,16 +5786,16 @@
         <v>8</v>
       </c>
       <c r="B319" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C319" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D319" s="3">
-        <v>314</v>
+        <v>281</v>
       </c>
       <c r="E319" s="3">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="320" spans="1:5">
@@ -5806,13 +5806,13 @@
         <v>2023</v>
       </c>
       <c r="C320" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D320" s="3">
-        <v>508</v>
+        <v>274</v>
       </c>
       <c r="E320" s="3">
-        <v>166</v>
+        <v>114</v>
       </c>
     </row>
     <row r="321" spans="1:5">
@@ -5823,13 +5823,13 @@
         <v>2023</v>
       </c>
       <c r="C321" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D321" s="3">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E321" s="3">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="322" spans="1:5">
@@ -5840,13 +5840,13 @@
         <v>2023</v>
       </c>
       <c r="C322" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D322" s="3">
-        <v>274</v>
+        <v>314</v>
       </c>
       <c r="E322" s="3">
-        <v>87</v>
+        <v>127</v>
       </c>
     </row>
     <row r="323" spans="1:5">
@@ -5857,13 +5857,13 @@
         <v>2023</v>
       </c>
       <c r="C323" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D323" s="3">
-        <v>257</v>
+        <v>508</v>
       </c>
       <c r="E323" s="3">
-        <v>88</v>
+        <v>166</v>
       </c>
     </row>
     <row r="324" spans="1:5">
@@ -5874,13 +5874,13 @@
         <v>2023</v>
       </c>
       <c r="C324" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D324" s="3">
-        <v>286</v>
+        <v>269</v>
       </c>
       <c r="E324" s="3">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="325" spans="1:5">
@@ -5891,13 +5891,13 @@
         <v>2023</v>
       </c>
       <c r="C325" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D325" s="3">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E325" s="3">
-        <v>112</v>
+        <v>87</v>
       </c>
     </row>
     <row r="326" spans="1:5">
@@ -5908,13 +5908,13 @@
         <v>2023</v>
       </c>
       <c r="C326" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D326" s="3">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="E326" s="3">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="327" spans="1:5">
@@ -5925,13 +5925,13 @@
         <v>2023</v>
       </c>
       <c r="C327" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D327" s="3">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="E327" s="3">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="328" spans="1:5">
@@ -5942,13 +5942,13 @@
         <v>2023</v>
       </c>
       <c r="C328" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D328" s="3">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E328" s="3">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="329" spans="1:5">
@@ -5956,16 +5956,16 @@
         <v>8</v>
       </c>
       <c r="B329" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C329" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D329" s="3">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="E329" s="3">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="330" spans="1:5">
@@ -5973,16 +5973,16 @@
         <v>8</v>
       </c>
       <c r="B330" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C330" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D330" s="3">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="E330" s="3">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="331" spans="1:5">
@@ -5990,16 +5990,16 @@
         <v>8</v>
       </c>
       <c r="B331" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C331" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D331" s="3">
-        <v>314</v>
+        <v>266</v>
       </c>
       <c r="E331" s="3">
-        <v>119</v>
+        <v>93</v>
       </c>
     </row>
     <row r="332" spans="1:5">
@@ -6010,13 +6010,13 @@
         <v>2024</v>
       </c>
       <c r="C332" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D332" s="3">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="E332" s="3">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="333" spans="1:5">
@@ -6027,13 +6027,13 @@
         <v>2024</v>
       </c>
       <c r="C333" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D333" s="3">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="E333" s="3">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="334" spans="1:5">
@@ -6044,13 +6044,13 @@
         <v>2024</v>
       </c>
       <c r="C334" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D334" s="3">
-        <v>253</v>
+        <v>314</v>
       </c>
       <c r="E334" s="3">
-        <v>99</v>
+        <v>119</v>
       </c>
     </row>
     <row r="335" spans="1:5">
@@ -6061,13 +6061,13 @@
         <v>2024</v>
       </c>
       <c r="C335" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D335" s="3">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="E335" s="3">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="336" spans="1:5">
@@ -6078,13 +6078,13 @@
         <v>2024</v>
       </c>
       <c r="C336" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D336" s="3">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="E336" s="3">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="337" spans="1:5">
@@ -6095,13 +6095,13 @@
         <v>2024</v>
       </c>
       <c r="C337" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D337" s="3">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="E337" s="3">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="338" spans="1:5">
@@ -6112,13 +6112,13 @@
         <v>2024</v>
       </c>
       <c r="C338" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D338" s="3">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E338" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="339" spans="1:5">
@@ -6129,13 +6129,13 @@
         <v>2024</v>
       </c>
       <c r="C339" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D339" s="3">
-        <v>216</v>
+        <v>254</v>
       </c>
       <c r="E339" s="3">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -6146,13 +6146,13 @@
         <v>2024</v>
       </c>
       <c r="C340" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D340" s="3">
-        <v>235</v>
+        <v>268</v>
       </c>
       <c r="E340" s="3">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="341" spans="1:5">
@@ -6160,16 +6160,16 @@
         <v>8</v>
       </c>
       <c r="B341" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C341" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D341" s="3">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="E341" s="3">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="342" spans="1:5">
@@ -6177,16 +6177,16 @@
         <v>8</v>
       </c>
       <c r="B342" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C342" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D342" s="3">
-        <v>244</v>
+        <v>216</v>
       </c>
       <c r="E342" s="3">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="343" spans="1:5">
@@ -6194,16 +6194,16 @@
         <v>8</v>
       </c>
       <c r="B343" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C343" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D343" s="3">
-        <v>296</v>
+        <v>235</v>
       </c>
       <c r="E343" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="344" spans="1:5">
@@ -6214,13 +6214,13 @@
         <v>2025</v>
       </c>
       <c r="C344" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D344" s="3">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="E344" s="3">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="345" spans="1:5">
@@ -6231,13 +6231,13 @@
         <v>2025</v>
       </c>
       <c r="C345" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D345" s="3">
-        <v>296</v>
+        <v>244</v>
       </c>
       <c r="E345" s="3">
-        <v>119</v>
+        <v>91</v>
       </c>
     </row>
     <row r="346" spans="1:5">
@@ -6248,13 +6248,13 @@
         <v>2025</v>
       </c>
       <c r="C346" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D346" s="3">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="E346" s="3">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="347" spans="1:5">
@@ -6265,13 +6265,13 @@
         <v>2025</v>
       </c>
       <c r="C347" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D347" s="3">
-        <v>255</v>
+        <v>296</v>
       </c>
       <c r="E347" s="3">
-        <v>92</v>
+        <v>113</v>
       </c>
     </row>
     <row r="348" spans="1:5">
@@ -6282,13 +6282,13 @@
         <v>2025</v>
       </c>
       <c r="C348" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D348" s="3">
-        <v>262</v>
+        <v>296</v>
       </c>
       <c r="E348" s="3">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="349" spans="1:5">
@@ -6299,13 +6299,13 @@
         <v>2025</v>
       </c>
       <c r="C349" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D349" s="3">
-        <v>248</v>
+        <v>286</v>
       </c>
       <c r="E349" s="3">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="350" spans="1:5">
@@ -6316,10 +6316,10 @@
         <v>2025</v>
       </c>
       <c r="C350" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D350" s="3">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="E350" s="3">
         <v>92</v>
@@ -6333,13 +6333,13 @@
         <v>2025</v>
       </c>
       <c r="C351" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D351" s="3">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="E351" s="3">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="352" spans="1:5">
@@ -6350,13 +6350,13 @@
         <v>2025</v>
       </c>
       <c r="C352" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D352" s="3">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E352" s="3">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="353" spans="1:5">
@@ -6364,16 +6364,16 @@
         <v>8</v>
       </c>
       <c r="B353" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C353" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D353" s="3">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="E353" s="3">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="354" spans="1:5">
@@ -6381,16 +6381,16 @@
         <v>8</v>
       </c>
       <c r="B354" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C354" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D354" s="3">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E354" s="3">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="355" spans="1:5">
@@ -6398,16 +6398,16 @@
         <v>8</v>
       </c>
       <c r="B355" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C355" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D355" s="3">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="E355" s="3">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="356" spans="1:5">
@@ -6418,13 +6418,13 @@
         <v>2026</v>
       </c>
       <c r="C356" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D356" s="3">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="E356" s="3">
-        <v>86</v>
+        <v>95</v>
       </c>
     </row>
     <row r="357" spans="1:5">
@@ -6435,13 +6435,81 @@
         <v>2026</v>
       </c>
       <c r="C357" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D357" s="3">
+        <v>252</v>
+      </c>
+      <c r="E357" s="3">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="358" spans="1:5">
+      <c r="A358" t="s">
+        <v>8</v>
+      </c>
+      <c r="B358" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C358" s="2">
+        <v>3</v>
+      </c>
+      <c r="D358" s="3">
+        <v>291</v>
+      </c>
+      <c r="E358" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="359" spans="1:5">
+      <c r="A359" t="s">
+        <v>8</v>
+      </c>
+      <c r="B359" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C359" s="2">
+        <v>4</v>
+      </c>
+      <c r="D359" s="3">
+        <v>268</v>
+      </c>
+      <c r="E359" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="360" spans="1:5">
+      <c r="A360" t="s">
+        <v>8</v>
+      </c>
+      <c r="B360" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C360" s="2">
+        <v>5</v>
+      </c>
+      <c r="D360" s="3">
         <v>296</v>
       </c>
-      <c r="E357" s="3">
+      <c r="E360" s="3">
         <v>97</v>
+      </c>
+    </row>
+    <row r="361" spans="1:5">
+      <c r="A361" t="s">
+        <v>8</v>
+      </c>
+      <c r="B361" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C361" s="2">
+        <v>6</v>
+      </c>
+      <c r="D361" s="3">
+        <v>265</v>
+      </c>
+      <c r="E361" s="3">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Carregando dados de julho/2026
</commit_message>
<xml_diff>
--- a/upload/partos-2025.xlsx
+++ b/upload/partos-2025.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24000" windowHeight="9600"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="9">
   <si>
     <t>unidade</t>
   </si>
@@ -372,7 +372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E361"/>
+  <dimension ref="A1:E365"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1729,7 +1729,7 @@
         <v>7</v>
       </c>
       <c r="D80" s="3">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E80" s="3">
         <v>84</v>
@@ -1865,10 +1865,10 @@
         <v>3</v>
       </c>
       <c r="D88" s="3">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E88" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -1924,19 +1924,19 @@
     </row>
     <row r="92" spans="1:5">
       <c r="A92" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B92" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C92" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D92" s="3">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="E92" s="3">
-        <v>72</v>
+        <v>64</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -1947,13 +1947,13 @@
         <v>2019</v>
       </c>
       <c r="C93" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D93" s="3">
-        <v>122</v>
+        <v>134</v>
       </c>
       <c r="E93" s="3">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -1964,13 +1964,13 @@
         <v>2019</v>
       </c>
       <c r="C94" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D94" s="3">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E94" s="3">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -1981,13 +1981,13 @@
         <v>2019</v>
       </c>
       <c r="C95" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D95" s="3">
-        <v>97</v>
+        <v>126</v>
       </c>
       <c r="E95" s="3">
-        <v>54</v>
+        <v>72</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -1998,13 +1998,13 @@
         <v>2019</v>
       </c>
       <c r="C96" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D96" s="3">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="E96" s="3">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2015,13 +2015,13 @@
         <v>2019</v>
       </c>
       <c r="C97" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D97" s="3">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="E97" s="3">
-        <v>69</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2032,13 +2032,13 @@
         <v>2019</v>
       </c>
       <c r="C98" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D98" s="3">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="E98" s="3">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2049,13 +2049,13 @@
         <v>2019</v>
       </c>
       <c r="C99" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D99" s="3">
-        <v>93</v>
+        <v>133</v>
       </c>
       <c r="E99" s="3">
-        <v>51</v>
+        <v>74</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2066,13 +2066,13 @@
         <v>2019</v>
       </c>
       <c r="C100" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D100" s="3">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="E100" s="3">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2083,13 +2083,13 @@
         <v>2019</v>
       </c>
       <c r="C101" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D101" s="3">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="E101" s="3">
-        <v>57</v>
+        <v>48</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2100,13 +2100,13 @@
         <v>2019</v>
       </c>
       <c r="C102" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D102" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E102" s="3">
-        <v>45</v>
+        <v>57</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2117,13 +2117,13 @@
         <v>2019</v>
       </c>
       <c r="C103" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D103" s="3">
-        <v>100</v>
+        <v>87</v>
       </c>
       <c r="E103" s="3">
-        <v>40</v>
+        <v>45</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2131,16 +2131,16 @@
         <v>6</v>
       </c>
       <c r="B104" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C104" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D104" s="3">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E104" s="3">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2151,13 +2151,13 @@
         <v>2020</v>
       </c>
       <c r="C105" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D105" s="3">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E105" s="3">
-        <v>48</v>
+        <v>42</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2168,13 +2168,13 @@
         <v>2020</v>
       </c>
       <c r="C106" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D106" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E106" s="3">
-        <v>70</v>
+        <v>48</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2185,13 +2185,13 @@
         <v>2020</v>
       </c>
       <c r="C107" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D107" s="3">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E107" s="3">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2202,13 +2202,13 @@
         <v>2020</v>
       </c>
       <c r="C108" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D108" s="3">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E108" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2219,13 +2219,13 @@
         <v>2020</v>
       </c>
       <c r="C109" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D109" s="3">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="E109" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2236,13 +2236,13 @@
         <v>2020</v>
       </c>
       <c r="C110" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D110" s="3">
-        <v>153</v>
+        <v>112</v>
       </c>
       <c r="E110" s="3">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2253,13 +2253,13 @@
         <v>2020</v>
       </c>
       <c r="C111" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D111" s="3">
-        <v>94</v>
+        <v>153</v>
       </c>
       <c r="E111" s="3">
-        <v>47</v>
+        <v>66</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2270,13 +2270,13 @@
         <v>2020</v>
       </c>
       <c r="C112" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D112" s="3">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="E112" s="3">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2287,13 +2287,13 @@
         <v>2020</v>
       </c>
       <c r="C113" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D113" s="3">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="E113" s="3">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2304,13 +2304,13 @@
         <v>2020</v>
       </c>
       <c r="C114" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D114" s="3">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="E114" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2321,13 +2321,13 @@
         <v>2020</v>
       </c>
       <c r="C115" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D115" s="3">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="E115" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2335,16 +2335,16 @@
         <v>6</v>
       </c>
       <c r="B116" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C116" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D116" s="3">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="E116" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2355,13 +2355,13 @@
         <v>2021</v>
       </c>
       <c r="C117" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D117" s="3">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="E117" s="3">
-        <v>70</v>
+        <v>50</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2372,13 +2372,13 @@
         <v>2021</v>
       </c>
       <c r="C118" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D118" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E118" s="3">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2389,13 +2389,13 @@
         <v>2021</v>
       </c>
       <c r="C119" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D119" s="3">
         <v>123</v>
       </c>
       <c r="E119" s="3">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2406,13 +2406,13 @@
         <v>2021</v>
       </c>
       <c r="C120" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D120" s="3">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E120" s="3">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2423,13 +2423,13 @@
         <v>2021</v>
       </c>
       <c r="C121" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D121" s="3">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="E121" s="3">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -2440,13 +2440,13 @@
         <v>2021</v>
       </c>
       <c r="C122" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D122" s="3">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E122" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -2457,13 +2457,13 @@
         <v>2021</v>
       </c>
       <c r="C123" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D123" s="3">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E123" s="3">
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -2474,10 +2474,10 @@
         <v>2021</v>
       </c>
       <c r="C124" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D124" s="3">
-        <v>115</v>
+        <v>134</v>
       </c>
       <c r="E124" s="3">
         <v>63</v>
@@ -2491,13 +2491,13 @@
         <v>2021</v>
       </c>
       <c r="C125" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D125" s="3">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E125" s="3">
-        <v>45</v>
+        <v>63</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2508,13 +2508,13 @@
         <v>2021</v>
       </c>
       <c r="C126" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D126" s="3">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="E126" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2525,13 +2525,13 @@
         <v>2021</v>
       </c>
       <c r="C127" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D127" s="3">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="E127" s="3">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2539,16 +2539,16 @@
         <v>6</v>
       </c>
       <c r="B128" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C128" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D128" s="3">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="E128" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2559,13 +2559,13 @@
         <v>2022</v>
       </c>
       <c r="C129" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D129" s="3">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E129" s="3">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -2576,13 +2576,13 @@
         <v>2022</v>
       </c>
       <c r="C130" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D130" s="3">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E130" s="3">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -2593,13 +2593,13 @@
         <v>2022</v>
       </c>
       <c r="C131" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D131" s="3">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="E131" s="3">
-        <v>52</v>
+        <v>69</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2610,10 +2610,10 @@
         <v>2022</v>
       </c>
       <c r="C132" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D132" s="3">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E132" s="3">
         <v>52</v>
@@ -2627,13 +2627,13 @@
         <v>2022</v>
       </c>
       <c r="C133" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D133" s="3">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E133" s="3">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2644,13 +2644,13 @@
         <v>2022</v>
       </c>
       <c r="C134" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D134" s="3">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="E134" s="3">
-        <v>39</v>
+        <v>54</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2661,13 +2661,13 @@
         <v>2022</v>
       </c>
       <c r="C135" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D135" s="3">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="E135" s="3">
-        <v>69</v>
+        <v>39</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2678,13 +2678,13 @@
         <v>2022</v>
       </c>
       <c r="C136" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D136" s="3">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="E136" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2695,13 +2695,13 @@
         <v>2022</v>
       </c>
       <c r="C137" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D137" s="3">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E137" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2712,13 +2712,13 @@
         <v>2022</v>
       </c>
       <c r="C138" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D138" s="3">
-        <v>118</v>
+        <v>96</v>
       </c>
       <c r="E138" s="3">
-        <v>72</v>
+        <v>52</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2729,13 +2729,13 @@
         <v>2022</v>
       </c>
       <c r="C139" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D139" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E139" s="3">
-        <v>58</v>
+        <v>72</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -2743,16 +2743,16 @@
         <v>6</v>
       </c>
       <c r="B140" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C140" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D140" s="3">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E140" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -2763,13 +2763,13 @@
         <v>2023</v>
       </c>
       <c r="C141" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D141" s="3">
-        <v>101</v>
+        <v>129</v>
       </c>
       <c r="E141" s="3">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -2780,13 +2780,13 @@
         <v>2023</v>
       </c>
       <c r="C142" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D142" s="3">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="E142" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -2797,13 +2797,13 @@
         <v>2023</v>
       </c>
       <c r="C143" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D143" s="3">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E143" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -2814,13 +2814,13 @@
         <v>2023</v>
       </c>
       <c r="C144" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D144" s="3">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="E144" s="3">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -2831,13 +2831,13 @@
         <v>2023</v>
       </c>
       <c r="C145" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D145" s="3">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="E145" s="3">
-        <v>73</v>
+        <v>59</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -2848,13 +2848,13 @@
         <v>2023</v>
       </c>
       <c r="C146" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D146" s="3">
-        <v>99</v>
+        <v>121</v>
       </c>
       <c r="E146" s="3">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -2865,13 +2865,13 @@
         <v>2023</v>
       </c>
       <c r="C147" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D147" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E147" s="3">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -2882,13 +2882,13 @@
         <v>2023</v>
       </c>
       <c r="C148" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D148" s="3">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="E148" s="3">
-        <v>69</v>
+        <v>57</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -2899,13 +2899,13 @@
         <v>2023</v>
       </c>
       <c r="C149" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D149" s="3">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="E149" s="3">
-        <v>59</v>
+        <v>69</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -2916,13 +2916,13 @@
         <v>2023</v>
       </c>
       <c r="C150" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D150" s="3">
-        <v>137</v>
+        <v>98</v>
       </c>
       <c r="E150" s="3">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -2933,13 +2933,13 @@
         <v>2023</v>
       </c>
       <c r="C151" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D151" s="3">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="E151" s="3">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -2947,16 +2947,16 @@
         <v>6</v>
       </c>
       <c r="B152" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C152" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D152" s="3">
-        <v>112</v>
+        <v>96</v>
       </c>
       <c r="E152" s="3">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -2967,13 +2967,13 @@
         <v>2024</v>
       </c>
       <c r="C153" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D153" s="3">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="E153" s="3">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -2984,13 +2984,13 @@
         <v>2024</v>
       </c>
       <c r="C154" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D154" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E154" s="3">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -3001,13 +3001,13 @@
         <v>2024</v>
       </c>
       <c r="C155" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D155" s="3">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="E155" s="3">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -3018,13 +3018,13 @@
         <v>2024</v>
       </c>
       <c r="C156" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D156" s="3">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="E156" s="3">
-        <v>72</v>
+        <v>59</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -3035,13 +3035,13 @@
         <v>2024</v>
       </c>
       <c r="C157" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D157" s="3">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="E157" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -3052,13 +3052,13 @@
         <v>2024</v>
       </c>
       <c r="C158" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D158" s="3">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="E158" s="3">
-        <v>42</v>
+        <v>64</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -3069,13 +3069,13 @@
         <v>2024</v>
       </c>
       <c r="C159" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D159" s="3">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E159" s="3">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -3086,13 +3086,13 @@
         <v>2024</v>
       </c>
       <c r="C160" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D160" s="3">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="E160" s="3">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -3103,13 +3103,13 @@
         <v>2024</v>
       </c>
       <c r="C161" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D161" s="3">
-        <v>101</v>
+        <v>113</v>
       </c>
       <c r="E161" s="3">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -3120,13 +3120,13 @@
         <v>2024</v>
       </c>
       <c r="C162" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D162" s="3">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="E162" s="3">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -3137,13 +3137,13 @@
         <v>2024</v>
       </c>
       <c r="C163" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D163" s="3">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="E163" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -3151,16 +3151,16 @@
         <v>6</v>
       </c>
       <c r="B164" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C164" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D164" s="3">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="E164" s="3">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -3171,13 +3171,13 @@
         <v>2025</v>
       </c>
       <c r="C165" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D165" s="3">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E165" s="3">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -3188,13 +3188,13 @@
         <v>2025</v>
       </c>
       <c r="C166" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D166" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E166" s="3">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -3205,13 +3205,13 @@
         <v>2025</v>
       </c>
       <c r="C167" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D167" s="3">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E167" s="3">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -3222,13 +3222,13 @@
         <v>2025</v>
       </c>
       <c r="C168" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D168" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E168" s="3">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -3239,13 +3239,13 @@
         <v>2025</v>
       </c>
       <c r="C169" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D169" s="3">
         <v>106</v>
       </c>
       <c r="E169" s="3">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -3256,13 +3256,13 @@
         <v>2025</v>
       </c>
       <c r="C170" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D170" s="3">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E170" s="3">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -3273,13 +3273,13 @@
         <v>2025</v>
       </c>
       <c r="C171" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D171" s="3">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="E171" s="3">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="172" spans="1:5">
@@ -3290,13 +3290,13 @@
         <v>2025</v>
       </c>
       <c r="C172" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D172" s="3">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E172" s="3">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="173" spans="1:5">
@@ -3307,13 +3307,13 @@
         <v>2025</v>
       </c>
       <c r="C173" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D173" s="3">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="E173" s="3">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="174" spans="1:5">
@@ -3324,13 +3324,13 @@
         <v>2025</v>
       </c>
       <c r="C174" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D174" s="3">
-        <v>115</v>
+        <v>106</v>
       </c>
       <c r="E174" s="3">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="175" spans="1:5">
@@ -3341,13 +3341,13 @@
         <v>2025</v>
       </c>
       <c r="C175" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D175" s="3">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="E175" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="176" spans="1:5">
@@ -3355,16 +3355,16 @@
         <v>6</v>
       </c>
       <c r="B176" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C176" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D176" s="3">
-        <v>117</v>
+        <v>95</v>
       </c>
       <c r="E176" s="3">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="177" spans="1:5">
@@ -3375,13 +3375,13 @@
         <v>2026</v>
       </c>
       <c r="C177" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D177" s="3">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E177" s="3">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="178" spans="1:5">
@@ -3392,13 +3392,13 @@
         <v>2026</v>
       </c>
       <c r="C178" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D178" s="3">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E178" s="3">
-        <v>52</v>
+        <v>62</v>
       </c>
     </row>
     <row r="179" spans="1:5">
@@ -3409,13 +3409,13 @@
         <v>2026</v>
       </c>
       <c r="C179" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D179" s="3">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="E179" s="3">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="180" spans="1:5">
@@ -3426,13 +3426,13 @@
         <v>2026</v>
       </c>
       <c r="C180" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D180" s="3">
-        <v>140</v>
+        <v>107</v>
       </c>
       <c r="E180" s="3">
-        <v>72</v>
+        <v>48</v>
       </c>
     </row>
     <row r="181" spans="1:5">
@@ -3443,47 +3443,47 @@
         <v>2026</v>
       </c>
       <c r="C181" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D181" s="3">
-        <v>53</v>
+        <v>140</v>
       </c>
       <c r="E181" s="3">
-        <v>34</v>
+        <v>72</v>
       </c>
     </row>
     <row r="182" spans="1:5">
       <c r="A182" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B182" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C182" s="2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D182" s="3">
-        <v>115</v>
+        <v>53</v>
       </c>
       <c r="E182" s="3">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="183" spans="1:5">
       <c r="A183" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B183" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C183" s="2">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D183" s="3">
-        <v>116</v>
+        <v>70</v>
       </c>
       <c r="E183" s="3">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="184" spans="1:5">
@@ -3494,13 +3494,13 @@
         <v>2019</v>
       </c>
       <c r="C184" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D184" s="3">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E184" s="3">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="185" spans="1:5">
@@ -3511,13 +3511,13 @@
         <v>2019</v>
       </c>
       <c r="C185" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D185" s="3">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="E185" s="3">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="186" spans="1:5">
@@ -3528,13 +3528,13 @@
         <v>2019</v>
       </c>
       <c r="C186" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D186" s="3">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E186" s="3">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="187" spans="1:5">
@@ -3545,13 +3545,13 @@
         <v>2019</v>
       </c>
       <c r="C187" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D187" s="3">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="E187" s="3">
-        <v>47</v>
+        <v>64</v>
       </c>
     </row>
     <row r="188" spans="1:5">
@@ -3562,13 +3562,13 @@
         <v>2019</v>
       </c>
       <c r="C188" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D188" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E188" s="3">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="189" spans="1:5">
@@ -3579,13 +3579,13 @@
         <v>2019</v>
       </c>
       <c r="C189" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D189" s="3">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="E189" s="3">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="190" spans="1:5">
@@ -3596,10 +3596,10 @@
         <v>2019</v>
       </c>
       <c r="C190" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D190" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E190" s="3">
         <v>50</v>
@@ -3613,13 +3613,13 @@
         <v>2019</v>
       </c>
       <c r="C191" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D191" s="3">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="E191" s="3">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="192" spans="1:5">
@@ -3630,13 +3630,13 @@
         <v>2019</v>
       </c>
       <c r="C192" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D192" s="3">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="E192" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="193" spans="1:5">
@@ -3647,13 +3647,13 @@
         <v>2019</v>
       </c>
       <c r="C193" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D193" s="3">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E193" s="3">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="194" spans="1:5">
@@ -3661,16 +3661,16 @@
         <v>7</v>
       </c>
       <c r="B194" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C194" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D194" s="3">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E194" s="3">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="195" spans="1:5">
@@ -3678,16 +3678,16 @@
         <v>7</v>
       </c>
       <c r="B195" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C195" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D195" s="3">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="E195" s="3">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="196" spans="1:5">
@@ -3698,13 +3698,13 @@
         <v>2020</v>
       </c>
       <c r="C196" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D196" s="3">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="E196" s="3">
-        <v>61</v>
+        <v>37</v>
       </c>
     </row>
     <row r="197" spans="1:5">
@@ -3715,13 +3715,13 @@
         <v>2020</v>
       </c>
       <c r="C197" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D197" s="3">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="E197" s="3">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="198" spans="1:5">
@@ -3732,13 +3732,13 @@
         <v>2020</v>
       </c>
       <c r="C198" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D198" s="3">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E198" s="3">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="199" spans="1:5">
@@ -3749,10 +3749,10 @@
         <v>2020</v>
       </c>
       <c r="C199" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D199" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="E199" s="3">
         <v>51</v>
@@ -3766,13 +3766,13 @@
         <v>2020</v>
       </c>
       <c r="C200" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D200" s="3">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="E200" s="3">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="201" spans="1:5">
@@ -3783,13 +3783,13 @@
         <v>2020</v>
       </c>
       <c r="C201" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D201" s="3">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="E201" s="3">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="202" spans="1:5">
@@ -3800,13 +3800,13 @@
         <v>2020</v>
       </c>
       <c r="C202" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D202" s="3">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E202" s="3">
-        <v>41</v>
+        <v>56</v>
       </c>
     </row>
     <row r="203" spans="1:5">
@@ -3817,13 +3817,13 @@
         <v>2020</v>
       </c>
       <c r="C203" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D203" s="3">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="E203" s="3">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="204" spans="1:5">
@@ -3834,13 +3834,13 @@
         <v>2020</v>
       </c>
       <c r="C204" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D204" s="3">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="E204" s="3">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="205" spans="1:5">
@@ -3851,13 +3851,13 @@
         <v>2020</v>
       </c>
       <c r="C205" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D205" s="3">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="E205" s="3">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="206" spans="1:5">
@@ -3865,16 +3865,16 @@
         <v>7</v>
       </c>
       <c r="B206" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C206" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D206" s="3">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E206" s="3">
-        <v>44</v>
+        <v>54</v>
       </c>
     </row>
     <row r="207" spans="1:5">
@@ -3882,13 +3882,13 @@
         <v>7</v>
       </c>
       <c r="B207" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C207" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D207" s="3">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E207" s="3">
         <v>44</v>
@@ -3902,13 +3902,13 @@
         <v>2021</v>
       </c>
       <c r="C208" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D208" s="3">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E208" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="209" spans="1:5">
@@ -3919,13 +3919,13 @@
         <v>2021</v>
       </c>
       <c r="C209" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D209" s="3">
-        <v>115</v>
+        <v>95</v>
       </c>
       <c r="E209" s="3">
-        <v>62</v>
+        <v>44</v>
       </c>
     </row>
     <row r="210" spans="1:5">
@@ -3936,13 +3936,13 @@
         <v>2021</v>
       </c>
       <c r="C210" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D210" s="3">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="E210" s="3">
-        <v>46</v>
+        <v>62</v>
       </c>
     </row>
     <row r="211" spans="1:5">
@@ -3953,13 +3953,13 @@
         <v>2021</v>
       </c>
       <c r="C211" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D211" s="3">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="E211" s="3">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="212" spans="1:5">
@@ -3970,13 +3970,13 @@
         <v>2021</v>
       </c>
       <c r="C212" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D212" s="3">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="E212" s="3">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="213" spans="1:5">
@@ -3987,13 +3987,13 @@
         <v>2021</v>
       </c>
       <c r="C213" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D213" s="3">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E213" s="3">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="214" spans="1:5">
@@ -4004,13 +4004,13 @@
         <v>2021</v>
       </c>
       <c r="C214" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D214" s="3">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="E214" s="3">
-        <v>46</v>
+        <v>53</v>
       </c>
     </row>
     <row r="215" spans="1:5">
@@ -4021,13 +4021,13 @@
         <v>2021</v>
       </c>
       <c r="C215" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D215" s="3">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="E215" s="3">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="216" spans="1:5">
@@ -4038,13 +4038,13 @@
         <v>2021</v>
       </c>
       <c r="C216" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D216" s="3">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="E216" s="3">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="217" spans="1:5">
@@ -4055,13 +4055,13 @@
         <v>2021</v>
       </c>
       <c r="C217" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D217" s="3">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E217" s="3">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="218" spans="1:5">
@@ -4069,16 +4069,16 @@
         <v>7</v>
       </c>
       <c r="B218" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C218" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D218" s="3">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E218" s="3">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="219" spans="1:5">
@@ -4086,16 +4086,16 @@
         <v>7</v>
       </c>
       <c r="B219" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C219" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D219" s="3">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="E219" s="3">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="220" spans="1:5">
@@ -4106,13 +4106,13 @@
         <v>2022</v>
       </c>
       <c r="C220" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D220" s="3">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="E220" s="3">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="221" spans="1:5">
@@ -4123,13 +4123,13 @@
         <v>2022</v>
       </c>
       <c r="C221" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D221" s="3">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="E221" s="3">
-        <v>59</v>
+        <v>51</v>
       </c>
     </row>
     <row r="222" spans="1:5">
@@ -4140,13 +4140,13 @@
         <v>2022</v>
       </c>
       <c r="C222" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D222" s="3">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E222" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="223" spans="1:5">
@@ -4157,13 +4157,13 @@
         <v>2022</v>
       </c>
       <c r="C223" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D223" s="3">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="E223" s="3">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="224" spans="1:5">
@@ -4174,13 +4174,13 @@
         <v>2022</v>
       </c>
       <c r="C224" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D224" s="3">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E224" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="225" spans="1:5">
@@ -4191,13 +4191,13 @@
         <v>2022</v>
       </c>
       <c r="C225" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D225" s="3">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E225" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="226" spans="1:5">
@@ -4208,13 +4208,13 @@
         <v>2022</v>
       </c>
       <c r="C226" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D226" s="3">
-        <v>104</v>
+        <v>118</v>
       </c>
       <c r="E226" s="3">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="227" spans="1:5">
@@ -4225,13 +4225,13 @@
         <v>2022</v>
       </c>
       <c r="C227" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D227" s="3">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="E227" s="3">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="228" spans="1:5">
@@ -4242,13 +4242,13 @@
         <v>2022</v>
       </c>
       <c r="C228" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D228" s="3">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="E228" s="3">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="229" spans="1:5">
@@ -4259,13 +4259,13 @@
         <v>2022</v>
       </c>
       <c r="C229" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D229" s="3">
-        <v>110</v>
+        <v>83</v>
       </c>
       <c r="E229" s="3">
-        <v>61</v>
+        <v>33</v>
       </c>
     </row>
     <row r="230" spans="1:5">
@@ -4273,16 +4273,16 @@
         <v>7</v>
       </c>
       <c r="B230" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C230" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D230" s="3">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="E230" s="3">
-        <v>54</v>
+        <v>38</v>
       </c>
     </row>
     <row r="231" spans="1:5">
@@ -4290,16 +4290,16 @@
         <v>7</v>
       </c>
       <c r="B231" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C231" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D231" s="3">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="E231" s="3">
-        <v>44</v>
+        <v>61</v>
       </c>
     </row>
     <row r="232" spans="1:5">
@@ -4310,13 +4310,13 @@
         <v>2023</v>
       </c>
       <c r="C232" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D232" s="3">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="E232" s="3">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="233" spans="1:5">
@@ -4327,13 +4327,13 @@
         <v>2023</v>
       </c>
       <c r="C233" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D233" s="3">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="E233" s="3">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="234" spans="1:5">
@@ -4344,13 +4344,13 @@
         <v>2023</v>
       </c>
       <c r="C234" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D234" s="3">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="E234" s="3">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="235" spans="1:5">
@@ -4361,13 +4361,13 @@
         <v>2023</v>
       </c>
       <c r="C235" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D235" s="3">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="E235" s="3">
-        <v>65</v>
+        <v>52</v>
       </c>
     </row>
     <row r="236" spans="1:5">
@@ -4378,13 +4378,13 @@
         <v>2023</v>
       </c>
       <c r="C236" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D236" s="3">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E236" s="3">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="237" spans="1:5">
@@ -4395,13 +4395,13 @@
         <v>2023</v>
       </c>
       <c r="C237" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D237" s="3">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="E237" s="3">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="238" spans="1:5">
@@ -4412,13 +4412,13 @@
         <v>2023</v>
       </c>
       <c r="C238" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D238" s="3">
-        <v>98</v>
+        <v>110</v>
       </c>
       <c r="E238" s="3">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="239" spans="1:5">
@@ -4429,13 +4429,13 @@
         <v>2023</v>
       </c>
       <c r="C239" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D239" s="3">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="E239" s="3">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="240" spans="1:5">
@@ -4446,10 +4446,10 @@
         <v>2023</v>
       </c>
       <c r="C240" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D240" s="3">
-        <v>120</v>
+        <v>98</v>
       </c>
       <c r="E240" s="3">
         <v>54</v>
@@ -4463,13 +4463,13 @@
         <v>2023</v>
       </c>
       <c r="C241" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D241" s="3">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="E241" s="3">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="242" spans="1:5">
@@ -4477,16 +4477,16 @@
         <v>7</v>
       </c>
       <c r="B242" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C242" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D242" s="3">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E242" s="3">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="243" spans="1:5">
@@ -4494,16 +4494,16 @@
         <v>7</v>
       </c>
       <c r="B243" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C243" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D243" s="3">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E243" s="3">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="244" spans="1:5">
@@ -4514,13 +4514,13 @@
         <v>2024</v>
       </c>
       <c r="C244" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D244" s="3">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="E244" s="3">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="245" spans="1:5">
@@ -4531,13 +4531,13 @@
         <v>2024</v>
       </c>
       <c r="C245" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D245" s="3">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="E245" s="3">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="246" spans="1:5">
@@ -4548,13 +4548,13 @@
         <v>2024</v>
       </c>
       <c r="C246" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D246" s="3">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="E246" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="247" spans="1:5">
@@ -4565,13 +4565,13 @@
         <v>2024</v>
       </c>
       <c r="C247" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D247" s="3">
-        <v>124</v>
+        <v>113</v>
       </c>
       <c r="E247" s="3">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="248" spans="1:5">
@@ -4582,13 +4582,13 @@
         <v>2024</v>
       </c>
       <c r="C248" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D248" s="3">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="E248" s="3">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="249" spans="1:5">
@@ -4599,13 +4599,13 @@
         <v>2024</v>
       </c>
       <c r="C249" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D249" s="3">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="E249" s="3">
-        <v>52</v>
+        <v>75</v>
       </c>
     </row>
     <row r="250" spans="1:5">
@@ -4616,13 +4616,13 @@
         <v>2024</v>
       </c>
       <c r="C250" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D250" s="3">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="E250" s="3">
-        <v>59</v>
+        <v>49</v>
       </c>
     </row>
     <row r="251" spans="1:5">
@@ -4633,13 +4633,13 @@
         <v>2024</v>
       </c>
       <c r="C251" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D251" s="3">
-        <v>118</v>
+        <v>101</v>
       </c>
       <c r="E251" s="3">
-        <v>62</v>
+        <v>52</v>
       </c>
     </row>
     <row r="252" spans="1:5">
@@ -4650,13 +4650,13 @@
         <v>2024</v>
       </c>
       <c r="C252" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D252" s="3">
-        <v>89</v>
+        <v>120</v>
       </c>
       <c r="E252" s="3">
-        <v>25</v>
+        <v>59</v>
       </c>
     </row>
     <row r="253" spans="1:5">
@@ -4667,13 +4667,13 @@
         <v>2024</v>
       </c>
       <c r="C253" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D253" s="3">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="E253" s="3">
-        <v>45</v>
+        <v>62</v>
       </c>
     </row>
     <row r="254" spans="1:5">
@@ -4681,16 +4681,16 @@
         <v>7</v>
       </c>
       <c r="B254" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C254" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D254" s="3">
-        <v>113</v>
+        <v>89</v>
       </c>
       <c r="E254" s="3">
-        <v>54</v>
+        <v>25</v>
       </c>
     </row>
     <row r="255" spans="1:5">
@@ -4698,16 +4698,16 @@
         <v>7</v>
       </c>
       <c r="B255" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C255" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D255" s="3">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="E255" s="3">
-        <v>53</v>
+        <v>45</v>
       </c>
     </row>
     <row r="256" spans="1:5">
@@ -4718,13 +4718,13 @@
         <v>2025</v>
       </c>
       <c r="C256" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D256" s="3">
-        <v>160</v>
+        <v>113</v>
       </c>
       <c r="E256" s="3">
-        <v>79</v>
+        <v>54</v>
       </c>
     </row>
     <row r="257" spans="1:5">
@@ -4735,13 +4735,13 @@
         <v>2025</v>
       </c>
       <c r="C257" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D257" s="3">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="E257" s="3">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="258" spans="1:5">
@@ -4752,13 +4752,13 @@
         <v>2025</v>
       </c>
       <c r="C258" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D258" s="3">
-        <v>139</v>
+        <v>160</v>
       </c>
       <c r="E258" s="3">
-        <v>71</v>
+        <v>79</v>
       </c>
     </row>
     <row r="259" spans="1:5">
@@ -4769,13 +4769,13 @@
         <v>2025</v>
       </c>
       <c r="C259" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D259" s="3">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="E259" s="3">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="260" spans="1:5">
@@ -4786,13 +4786,13 @@
         <v>2025</v>
       </c>
       <c r="C260" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D260" s="3">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="E260" s="3">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="261" spans="1:5">
@@ -4803,13 +4803,13 @@
         <v>2025</v>
       </c>
       <c r="C261" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D261" s="3">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="E261" s="3">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="262" spans="1:5">
@@ -4820,13 +4820,13 @@
         <v>2025</v>
       </c>
       <c r="C262" s="2">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D262" s="3">
-        <v>108</v>
+        <v>131</v>
       </c>
       <c r="E262" s="3">
-        <v>54</v>
+        <v>69</v>
       </c>
     </row>
     <row r="263" spans="1:5">
@@ -4837,13 +4837,13 @@
         <v>2025</v>
       </c>
       <c r="C263" s="2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D263" s="3">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="E263" s="3">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="264" spans="1:5">
@@ -4854,13 +4854,13 @@
         <v>2025</v>
       </c>
       <c r="C264" s="2">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D264" s="3">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="E264" s="3">
-        <v>65</v>
+        <v>54</v>
       </c>
     </row>
     <row r="265" spans="1:5">
@@ -4871,13 +4871,13 @@
         <v>2025</v>
       </c>
       <c r="C265" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D265" s="3">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="E265" s="3">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="266" spans="1:5">
@@ -4885,16 +4885,16 @@
         <v>7</v>
       </c>
       <c r="B266" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C266" s="2">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D266" s="3">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="E266" s="3">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="267" spans="1:5">
@@ -4902,16 +4902,16 @@
         <v>7</v>
       </c>
       <c r="B267" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C267" s="2">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D267" s="3">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="E267" s="3">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="268" spans="1:5">
@@ -4922,10 +4922,10 @@
         <v>2026</v>
       </c>
       <c r="C268" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D268" s="3">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="E268" s="3">
         <v>67</v>
@@ -4939,13 +4939,13 @@
         <v>2026</v>
       </c>
       <c r="C269" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D269" s="3">
-        <v>155</v>
+        <v>128</v>
       </c>
       <c r="E269" s="3">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
     <row r="270" spans="1:5">
@@ -4956,13 +4956,13 @@
         <v>2026</v>
       </c>
       <c r="C270" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D270" s="3">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E270" s="3">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="271" spans="1:5">
@@ -4973,64 +4973,64 @@
         <v>2026</v>
       </c>
       <c r="C271" s="2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D271" s="3">
-        <v>119</v>
+        <v>155</v>
       </c>
       <c r="E271" s="3">
-        <v>66</v>
+        <v>85</v>
       </c>
     </row>
     <row r="272" spans="1:5">
       <c r="A272" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B272" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C272" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D272" s="3">
-        <v>309</v>
+        <v>127</v>
       </c>
       <c r="E272" s="3">
-        <v>101</v>
+        <v>61</v>
       </c>
     </row>
     <row r="273" spans="1:5">
       <c r="A273" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B273" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C273" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D273" s="3">
-        <v>249</v>
+        <v>119</v>
       </c>
       <c r="E273" s="3">
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="274" spans="1:5">
       <c r="A274" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B274" s="2">
-        <v>2019</v>
+        <v>2026</v>
       </c>
       <c r="C274" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D274" s="3">
-        <v>298</v>
+        <v>142</v>
       </c>
       <c r="E274" s="3">
-        <v>93</v>
+        <v>72</v>
       </c>
     </row>
     <row r="275" spans="1:5">
@@ -5041,13 +5041,13 @@
         <v>2019</v>
       </c>
       <c r="C275" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D275" s="3">
-        <v>281</v>
+        <v>309</v>
       </c>
       <c r="E275" s="3">
-        <v>86</v>
+        <v>101</v>
       </c>
     </row>
     <row r="276" spans="1:5">
@@ -5058,13 +5058,13 @@
         <v>2019</v>
       </c>
       <c r="C276" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D276" s="3">
-        <v>296</v>
+        <v>249</v>
       </c>
       <c r="E276" s="3">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="277" spans="1:5">
@@ -5075,13 +5075,13 @@
         <v>2019</v>
       </c>
       <c r="C277" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D277" s="3">
-        <v>253</v>
+        <v>298</v>
       </c>
       <c r="E277" s="3">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="278" spans="1:5">
@@ -5092,13 +5092,13 @@
         <v>2019</v>
       </c>
       <c r="C278" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D278" s="3">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="E278" s="3">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="279" spans="1:5">
@@ -5109,13 +5109,13 @@
         <v>2019</v>
       </c>
       <c r="C279" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D279" s="3">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="E279" s="3">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="280" spans="1:5">
@@ -5126,13 +5126,13 @@
         <v>2019</v>
       </c>
       <c r="C280" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D280" s="3">
-        <v>277</v>
+        <v>253</v>
       </c>
       <c r="E280" s="3">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="281" spans="1:5">
@@ -5143,13 +5143,13 @@
         <v>2019</v>
       </c>
       <c r="C281" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D281" s="3">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E281" s="3">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="282" spans="1:5">
@@ -5160,13 +5160,13 @@
         <v>2019</v>
       </c>
       <c r="C282" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D282" s="3">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="E282" s="3">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="283" spans="1:5">
@@ -5177,13 +5177,13 @@
         <v>2019</v>
       </c>
       <c r="C283" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D283" s="3">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="E283" s="3">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="284" spans="1:5">
@@ -5191,16 +5191,16 @@
         <v>8</v>
       </c>
       <c r="B284" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C284" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D284" s="3">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="E284" s="3">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="285" spans="1:5">
@@ -5208,16 +5208,16 @@
         <v>8</v>
       </c>
       <c r="B285" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C285" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D285" s="3">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="E285" s="3">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="286" spans="1:5">
@@ -5225,16 +5225,16 @@
         <v>8</v>
       </c>
       <c r="B286" s="2">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="C286" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D286" s="3">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="E286" s="3">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="287" spans="1:5">
@@ -5245,13 +5245,13 @@
         <v>2020</v>
       </c>
       <c r="C287" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D287" s="3">
-        <v>283</v>
+        <v>257</v>
       </c>
       <c r="E287" s="3">
-        <v>101</v>
+        <v>72</v>
       </c>
     </row>
     <row r="288" spans="1:5">
@@ -5262,13 +5262,13 @@
         <v>2020</v>
       </c>
       <c r="C288" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D288" s="3">
-        <v>305</v>
+        <v>261</v>
       </c>
       <c r="E288" s="3">
-        <v>112</v>
+        <v>72</v>
       </c>
     </row>
     <row r="289" spans="1:5">
@@ -5279,13 +5279,13 @@
         <v>2020</v>
       </c>
       <c r="C289" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D289" s="3">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="E289" s="3">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="290" spans="1:5">
@@ -5296,13 +5296,13 @@
         <v>2020</v>
       </c>
       <c r="C290" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D290" s="3">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E290" s="3">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="291" spans="1:5">
@@ -5313,13 +5313,13 @@
         <v>2020</v>
       </c>
       <c r="C291" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D291" s="3">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="E291" s="3">
-        <v>74</v>
+        <v>112</v>
       </c>
     </row>
     <row r="292" spans="1:5">
@@ -5330,13 +5330,13 @@
         <v>2020</v>
       </c>
       <c r="C292" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D292" s="3">
-        <v>269</v>
+        <v>285</v>
       </c>
       <c r="E292" s="3">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="293" spans="1:5">
@@ -5347,10 +5347,10 @@
         <v>2020</v>
       </c>
       <c r="C293" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D293" s="3">
-        <v>247</v>
+        <v>281</v>
       </c>
       <c r="E293" s="3">
         <v>77</v>
@@ -5364,13 +5364,13 @@
         <v>2020</v>
       </c>
       <c r="C294" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D294" s="3">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="E294" s="3">
-        <v>92</v>
+        <v>74</v>
       </c>
     </row>
     <row r="295" spans="1:5">
@@ -5381,13 +5381,13 @@
         <v>2020</v>
       </c>
       <c r="C295" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D295" s="3">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="E295" s="3">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="296" spans="1:5">
@@ -5395,16 +5395,16 @@
         <v>8</v>
       </c>
       <c r="B296" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C296" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D296" s="3">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="E296" s="3">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="297" spans="1:5">
@@ -5412,16 +5412,16 @@
         <v>8</v>
       </c>
       <c r="B297" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C297" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D297" s="3">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="E297" s="3">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="298" spans="1:5">
@@ -5429,16 +5429,16 @@
         <v>8</v>
       </c>
       <c r="B298" s="2">
-        <v>2021</v>
+        <v>2020</v>
       </c>
       <c r="C298" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D298" s="3">
-        <v>289</v>
+        <v>260</v>
       </c>
       <c r="E298" s="3">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="299" spans="1:5">
@@ -5449,13 +5449,13 @@
         <v>2021</v>
       </c>
       <c r="C299" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D299" s="3">
-        <v>294</v>
+        <v>255</v>
       </c>
       <c r="E299" s="3">
-        <v>93</v>
+        <v>80</v>
       </c>
     </row>
     <row r="300" spans="1:5">
@@ -5466,13 +5466,13 @@
         <v>2021</v>
       </c>
       <c r="C300" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D300" s="3">
-        <v>318</v>
+        <v>257</v>
       </c>
       <c r="E300" s="3">
-        <v>108</v>
+        <v>89</v>
       </c>
     </row>
     <row r="301" spans="1:5">
@@ -5483,13 +5483,13 @@
         <v>2021</v>
       </c>
       <c r="C301" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D301" s="3">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="E301" s="3">
-        <v>100</v>
+        <v>84</v>
       </c>
     </row>
     <row r="302" spans="1:5">
@@ -5500,13 +5500,13 @@
         <v>2021</v>
       </c>
       <c r="C302" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D302" s="3">
         <v>294</v>
       </c>
       <c r="E302" s="3">
-        <v>99</v>
+        <v>93</v>
       </c>
     </row>
     <row r="303" spans="1:5">
@@ -5517,13 +5517,13 @@
         <v>2021</v>
       </c>
       <c r="C303" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D303" s="3">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="E303" s="3">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="304" spans="1:5">
@@ -5534,13 +5534,13 @@
         <v>2021</v>
       </c>
       <c r="C304" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D304" s="3">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="E304" s="3">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="305" spans="1:5">
@@ -5551,13 +5551,13 @@
         <v>2021</v>
       </c>
       <c r="C305" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D305" s="3">
-        <v>236</v>
+        <v>294</v>
       </c>
       <c r="E305" s="3">
-        <v>73</v>
+        <v>99</v>
       </c>
     </row>
     <row r="306" spans="1:5">
@@ -5568,13 +5568,13 @@
         <v>2021</v>
       </c>
       <c r="C306" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D306" s="3">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="E306" s="3">
-        <v>78</v>
+        <v>107</v>
       </c>
     </row>
     <row r="307" spans="1:5">
@@ -5585,13 +5585,13 @@
         <v>2021</v>
       </c>
       <c r="C307" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D307" s="3">
-        <v>235</v>
+        <v>277</v>
       </c>
       <c r="E307" s="3">
-        <v>73</v>
+        <v>102</v>
       </c>
     </row>
     <row r="308" spans="1:5">
@@ -5599,16 +5599,16 @@
         <v>8</v>
       </c>
       <c r="B308" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C308" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D308" s="3">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="E308" s="3">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="309" spans="1:5">
@@ -5616,16 +5616,16 @@
         <v>8</v>
       </c>
       <c r="B309" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C309" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D309" s="3">
-        <v>224</v>
+        <v>269</v>
       </c>
       <c r="E309" s="3">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="310" spans="1:5">
@@ -5633,16 +5633,16 @@
         <v>8</v>
       </c>
       <c r="B310" s="2">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="C310" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D310" s="3">
-        <v>278</v>
+        <v>235</v>
       </c>
       <c r="E310" s="3">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="311" spans="1:5">
@@ -5653,13 +5653,13 @@
         <v>2022</v>
       </c>
       <c r="C311" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D311" s="3">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="E311" s="3">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="312" spans="1:5">
@@ -5670,13 +5670,13 @@
         <v>2022</v>
       </c>
       <c r="C312" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D312" s="3">
-        <v>277</v>
+        <v>224</v>
       </c>
       <c r="E312" s="3">
-        <v>88</v>
+        <v>71</v>
       </c>
     </row>
     <row r="313" spans="1:5">
@@ -5687,13 +5687,13 @@
         <v>2022</v>
       </c>
       <c r="C313" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D313" s="3">
-        <v>253</v>
+        <v>278</v>
       </c>
       <c r="E313" s="3">
-        <v>73</v>
+        <v>83</v>
       </c>
     </row>
     <row r="314" spans="1:5">
@@ -5704,13 +5704,13 @@
         <v>2022</v>
       </c>
       <c r="C314" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D314" s="3">
-        <v>265</v>
+        <v>236</v>
       </c>
       <c r="E314" s="3">
-        <v>92</v>
+        <v>64</v>
       </c>
     </row>
     <row r="315" spans="1:5">
@@ -5721,13 +5721,13 @@
         <v>2022</v>
       </c>
       <c r="C315" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D315" s="3">
-        <v>239</v>
+        <v>277</v>
       </c>
       <c r="E315" s="3">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="316" spans="1:5">
@@ -5738,13 +5738,13 @@
         <v>2022</v>
       </c>
       <c r="C316" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D316" s="3">
-        <v>237</v>
+        <v>253</v>
       </c>
       <c r="E316" s="3">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="317" spans="1:5">
@@ -5755,13 +5755,13 @@
         <v>2022</v>
       </c>
       <c r="C317" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D317" s="3">
-        <v>236</v>
+        <v>265</v>
       </c>
       <c r="E317" s="3">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="318" spans="1:5">
@@ -5772,13 +5772,13 @@
         <v>2022</v>
       </c>
       <c r="C318" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D318" s="3">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E318" s="3">
-        <v>103</v>
+        <v>81</v>
       </c>
     </row>
     <row r="319" spans="1:5">
@@ -5789,13 +5789,13 @@
         <v>2022</v>
       </c>
       <c r="C319" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D319" s="3">
-        <v>281</v>
+        <v>237</v>
       </c>
       <c r="E319" s="3">
-        <v>97</v>
+        <v>80</v>
       </c>
     </row>
     <row r="320" spans="1:5">
@@ -5803,16 +5803,16 @@
         <v>8</v>
       </c>
       <c r="B320" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C320" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D320" s="3">
-        <v>274</v>
+        <v>236</v>
       </c>
       <c r="E320" s="3">
-        <v>114</v>
+        <v>93</v>
       </c>
     </row>
     <row r="321" spans="1:5">
@@ -5820,16 +5820,16 @@
         <v>8</v>
       </c>
       <c r="B321" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C321" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D321" s="3">
-        <v>270</v>
+        <v>245</v>
       </c>
       <c r="E321" s="3">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="322" spans="1:5">
@@ -5837,16 +5837,16 @@
         <v>8</v>
       </c>
       <c r="B322" s="2">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="C322" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D322" s="3">
-        <v>314</v>
+        <v>281</v>
       </c>
       <c r="E322" s="3">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="323" spans="1:5">
@@ -5857,13 +5857,13 @@
         <v>2023</v>
       </c>
       <c r="C323" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D323" s="3">
-        <v>508</v>
+        <v>274</v>
       </c>
       <c r="E323" s="3">
-        <v>166</v>
+        <v>114</v>
       </c>
     </row>
     <row r="324" spans="1:5">
@@ -5874,13 +5874,13 @@
         <v>2023</v>
       </c>
       <c r="C324" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D324" s="3">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E324" s="3">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="325" spans="1:5">
@@ -5891,13 +5891,13 @@
         <v>2023</v>
       </c>
       <c r="C325" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D325" s="3">
-        <v>274</v>
+        <v>314</v>
       </c>
       <c r="E325" s="3">
-        <v>87</v>
+        <v>127</v>
       </c>
     </row>
     <row r="326" spans="1:5">
@@ -5908,13 +5908,13 @@
         <v>2023</v>
       </c>
       <c r="C326" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D326" s="3">
-        <v>257</v>
+        <v>508</v>
       </c>
       <c r="E326" s="3">
-        <v>88</v>
+        <v>166</v>
       </c>
     </row>
     <row r="327" spans="1:5">
@@ -5925,13 +5925,13 @@
         <v>2023</v>
       </c>
       <c r="C327" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D327" s="3">
-        <v>286</v>
+        <v>269</v>
       </c>
       <c r="E327" s="3">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="328" spans="1:5">
@@ -5942,13 +5942,13 @@
         <v>2023</v>
       </c>
       <c r="C328" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D328" s="3">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="E328" s="3">
-        <v>112</v>
+        <v>87</v>
       </c>
     </row>
     <row r="329" spans="1:5">
@@ -5959,13 +5959,13 @@
         <v>2023</v>
       </c>
       <c r="C329" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D329" s="3">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="E329" s="3">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="330" spans="1:5">
@@ -5976,13 +5976,13 @@
         <v>2023</v>
       </c>
       <c r="C330" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D330" s="3">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="E330" s="3">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="331" spans="1:5">
@@ -5993,13 +5993,13 @@
         <v>2023</v>
       </c>
       <c r="C331" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D331" s="3">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="E331" s="3">
-        <v>93</v>
+        <v>112</v>
       </c>
     </row>
     <row r="332" spans="1:5">
@@ -6007,16 +6007,16 @@
         <v>8</v>
       </c>
       <c r="B332" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C332" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D332" s="3">
-        <v>249</v>
+        <v>266</v>
       </c>
       <c r="E332" s="3">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="333" spans="1:5">
@@ -6024,16 +6024,16 @@
         <v>8</v>
       </c>
       <c r="B333" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C333" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D333" s="3">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="E333" s="3">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="334" spans="1:5">
@@ -6041,16 +6041,16 @@
         <v>8</v>
       </c>
       <c r="B334" s="2">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="C334" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D334" s="3">
-        <v>314</v>
+        <v>266</v>
       </c>
       <c r="E334" s="3">
-        <v>119</v>
+        <v>93</v>
       </c>
     </row>
     <row r="335" spans="1:5">
@@ -6061,13 +6061,13 @@
         <v>2024</v>
       </c>
       <c r="C335" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D335" s="3">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="E335" s="3">
-        <v>96</v>
+        <v>88</v>
       </c>
     </row>
     <row r="336" spans="1:5">
@@ -6078,13 +6078,13 @@
         <v>2024</v>
       </c>
       <c r="C336" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D336" s="3">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="E336" s="3">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="337" spans="1:5">
@@ -6095,13 +6095,13 @@
         <v>2024</v>
       </c>
       <c r="C337" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D337" s="3">
-        <v>253</v>
+        <v>314</v>
       </c>
       <c r="E337" s="3">
-        <v>99</v>
+        <v>119</v>
       </c>
     </row>
     <row r="338" spans="1:5">
@@ -6112,13 +6112,13 @@
         <v>2024</v>
       </c>
       <c r="C338" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D338" s="3">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="E338" s="3">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="339" spans="1:5">
@@ -6129,13 +6129,13 @@
         <v>2024</v>
       </c>
       <c r="C339" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D339" s="3">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="E339" s="3">
-        <v>102</v>
+        <v>116</v>
       </c>
     </row>
     <row r="340" spans="1:5">
@@ -6146,13 +6146,13 @@
         <v>2024</v>
       </c>
       <c r="C340" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D340" s="3">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="E340" s="3">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="341" spans="1:5">
@@ -6163,13 +6163,13 @@
         <v>2024</v>
       </c>
       <c r="C341" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D341" s="3">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="E341" s="3">
-        <v>109</v>
+        <v>90</v>
       </c>
     </row>
     <row r="342" spans="1:5">
@@ -6180,13 +6180,13 @@
         <v>2024</v>
       </c>
       <c r="C342" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D342" s="3">
-        <v>216</v>
+        <v>254</v>
       </c>
       <c r="E342" s="3">
-        <v>82</v>
+        <v>102</v>
       </c>
     </row>
     <row r="343" spans="1:5">
@@ -6197,13 +6197,13 @@
         <v>2024</v>
       </c>
       <c r="C343" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D343" s="3">
-        <v>235</v>
+        <v>268</v>
       </c>
       <c r="E343" s="3">
-        <v>97</v>
+        <v>107</v>
       </c>
     </row>
     <row r="344" spans="1:5">
@@ -6211,16 +6211,16 @@
         <v>8</v>
       </c>
       <c r="B344" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C344" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D344" s="3">
-        <v>282</v>
+        <v>254</v>
       </c>
       <c r="E344" s="3">
-        <v>106</v>
+        <v>109</v>
       </c>
     </row>
     <row r="345" spans="1:5">
@@ -6228,16 +6228,16 @@
         <v>8</v>
       </c>
       <c r="B345" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C345" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D345" s="3">
-        <v>244</v>
+        <v>216</v>
       </c>
       <c r="E345" s="3">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="346" spans="1:5">
@@ -6245,16 +6245,16 @@
         <v>8</v>
       </c>
       <c r="B346" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C346" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D346" s="3">
-        <v>296</v>
+        <v>235</v>
       </c>
       <c r="E346" s="3">
-        <v>113</v>
+        <v>97</v>
       </c>
     </row>
     <row r="347" spans="1:5">
@@ -6265,13 +6265,13 @@
         <v>2025</v>
       </c>
       <c r="C347" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D347" s="3">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="E347" s="3">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="348" spans="1:5">
@@ -6282,13 +6282,13 @@
         <v>2025</v>
       </c>
       <c r="C348" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D348" s="3">
-        <v>296</v>
+        <v>244</v>
       </c>
       <c r="E348" s="3">
-        <v>119</v>
+        <v>91</v>
       </c>
     </row>
     <row r="349" spans="1:5">
@@ -6299,13 +6299,13 @@
         <v>2025</v>
       </c>
       <c r="C349" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D349" s="3">
-        <v>286</v>
+        <v>296</v>
       </c>
       <c r="E349" s="3">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
     <row r="350" spans="1:5">
@@ -6316,13 +6316,13 @@
         <v>2025</v>
       </c>
       <c r="C350" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D350" s="3">
-        <v>255</v>
+        <v>296</v>
       </c>
       <c r="E350" s="3">
-        <v>92</v>
+        <v>113</v>
       </c>
     </row>
     <row r="351" spans="1:5">
@@ -6333,13 +6333,13 @@
         <v>2025</v>
       </c>
       <c r="C351" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D351" s="3">
-        <v>262</v>
+        <v>296</v>
       </c>
       <c r="E351" s="3">
-        <v>97</v>
+        <v>119</v>
       </c>
     </row>
     <row r="352" spans="1:5">
@@ -6350,13 +6350,13 @@
         <v>2025</v>
       </c>
       <c r="C352" s="2">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D352" s="3">
-        <v>248</v>
+        <v>286</v>
       </c>
       <c r="E352" s="3">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="353" spans="1:5">
@@ -6367,10 +6367,10 @@
         <v>2025</v>
       </c>
       <c r="C353" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D353" s="3">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="E353" s="3">
         <v>92</v>
@@ -6384,13 +6384,13 @@
         <v>2025</v>
       </c>
       <c r="C354" s="2">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D354" s="3">
-        <v>246</v>
+        <v>262</v>
       </c>
       <c r="E354" s="3">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="355" spans="1:5">
@@ -6401,13 +6401,13 @@
         <v>2025</v>
       </c>
       <c r="C355" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D355" s="3">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E355" s="3">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="356" spans="1:5">
@@ -6415,16 +6415,16 @@
         <v>8</v>
       </c>
       <c r="B356" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C356" s="2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D356" s="3">
-        <v>250</v>
+        <v>266</v>
       </c>
       <c r="E356" s="3">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="357" spans="1:5">
@@ -6432,16 +6432,16 @@
         <v>8</v>
       </c>
       <c r="B357" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C357" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D357" s="3">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E357" s="3">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="358" spans="1:5">
@@ -6449,16 +6449,16 @@
         <v>8</v>
       </c>
       <c r="B358" s="2">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C358" s="2">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D358" s="3">
-        <v>291</v>
+        <v>250</v>
       </c>
       <c r="E358" s="3">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="359" spans="1:5">
@@ -6469,13 +6469,13 @@
         <v>2026</v>
       </c>
       <c r="C359" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D359" s="3">
-        <v>268</v>
+        <v>250</v>
       </c>
       <c r="E359" s="3">
-        <v>86</v>
+        <v>95</v>
       </c>
     </row>
     <row r="360" spans="1:5">
@@ -6486,13 +6486,13 @@
         <v>2026</v>
       </c>
       <c r="C360" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D360" s="3">
-        <v>296</v>
+        <v>252</v>
       </c>
       <c r="E360" s="3">
-        <v>97</v>
+        <v>82</v>
       </c>
     </row>
     <row r="361" spans="1:5">
@@ -6503,13 +6503,81 @@
         <v>2026</v>
       </c>
       <c r="C361" s="2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D361" s="3">
+        <v>291</v>
+      </c>
+      <c r="E361" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="362" spans="1:5">
+      <c r="A362" t="s">
+        <v>8</v>
+      </c>
+      <c r="B362" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C362" s="2">
+        <v>4</v>
+      </c>
+      <c r="D362" s="3">
+        <v>269</v>
+      </c>
+      <c r="E362" s="3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="363" spans="1:5">
+      <c r="A363" t="s">
+        <v>8</v>
+      </c>
+      <c r="B363" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C363" s="2">
+        <v>5</v>
+      </c>
+      <c r="D363" s="3">
+        <v>296</v>
+      </c>
+      <c r="E363" s="3">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="364" spans="1:5">
+      <c r="A364" t="s">
+        <v>8</v>
+      </c>
+      <c r="B364" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C364" s="2">
+        <v>6</v>
+      </c>
+      <c r="D364" s="3">
         <v>265</v>
       </c>
-      <c r="E361" s="3">
+      <c r="E364" s="3">
         <v>93</v>
+      </c>
+    </row>
+    <row r="365" spans="1:5">
+      <c r="A365" t="s">
+        <v>8</v>
+      </c>
+      <c r="B365" s="2">
+        <v>2026</v>
+      </c>
+      <c r="C365" s="2">
+        <v>7</v>
+      </c>
+      <c r="D365" s="3">
+        <v>259</v>
+      </c>
+      <c r="E365" s="3">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>